<commit_message>
fix: group VIX/TNX change columns and guard window formulas
</commit_message>
<xml_diff>
--- a/04_结果/示例审批/外部数据新版式示例.xlsx
+++ b/04_结果/示例审批/外部数据新版式示例.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -490,21 +490,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1. VIX/TNX 按 ETF 格式展示：第14行=名称，第15行=Open/High/Low/Close/Adj Close/Volume/回报。</t>
+          <t>1. VIX/TNX 原始数据按 ETF 格式展示：第14行=名称，第15行=Open/High/Low/Close/Adj Close/Volume。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2. 派生外部列：第14行=指标名称，第15行=计算公式（谁减谁），数据区为 Excel 公式。</t>
+          <t>2. VIX/TNX 回报与变化指标集中放一起，第15行直接写名称（如 VIX回报、VIX_Chg%、TNX_ChgBp），后面用空列分隔。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3. ETF 回报、VIX/TNX 回报、派生指标均用公式计算，回报率保留4位小数。</t>
+          <t>3. 其他派生外部列：第14行=指标名称，第15行=计算公式（谁减谁），数据区为 Excel 公式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4. ETF 回报、VIX/TNX 回报、派生指标均用公式计算，回报率保留4位小数。</t>
         </is>
       </c>
     </row>
@@ -519,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A14:CV42"/>
+  <dimension ref="A14:CW42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -622,6 +629,7 @@
     <col width="14" customWidth="1" min="98" max="98"/>
     <col width="14" customWidth="1" min="99" max="99"/>
     <col width="14" customWidth="1" min="100" max="100"/>
+    <col width="14" customWidth="1" min="101" max="101"/>
   </cols>
   <sheetData>
     <row r="14" ht="30" customHeight="1">
@@ -751,68 +759,53 @@
       <c r="CB14" s="2" t="n"/>
       <c r="CC14" s="2" t="n"/>
       <c r="CD14" s="2" t="n"/>
-      <c r="CE14" s="2" t="n"/>
-      <c r="CF14" s="2" t="inlineStr">
+      <c r="CE14" s="2" t="inlineStr">
         <is>
           <t>TNX</t>
         </is>
       </c>
+      <c r="CF14" s="2" t="n"/>
       <c r="CG14" s="2" t="n"/>
       <c r="CH14" s="2" t="n"/>
       <c r="CI14" s="2" t="n"/>
       <c r="CJ14" s="2" t="n"/>
       <c r="CK14" s="2" t="n"/>
-      <c r="CL14" s="2" t="inlineStr">
-        <is>
-          <t>VIX_Chg%</t>
-        </is>
-      </c>
-      <c r="CM14" s="2" t="inlineStr">
-        <is>
-          <t>TNX_ChgBp</t>
-        </is>
-      </c>
-      <c r="CN14" s="2" t="inlineStr">
-        <is>
-          <t>VIX_5dChg</t>
-        </is>
-      </c>
-      <c r="CO14" s="2" t="inlineStr">
-        <is>
-          <t>VIX_20dVol</t>
-        </is>
-      </c>
-      <c r="CP14" s="2" t="inlineStr">
+      <c r="CL14" s="2" t="n"/>
+      <c r="CM14" s="2" t="n"/>
+      <c r="CN14" s="2" t="n"/>
+      <c r="CO14" s="2" t="n"/>
+      <c r="CP14" s="2" t="n"/>
+      <c r="CQ14" s="2" t="inlineStr">
         <is>
           <t>CreditSpread</t>
         </is>
       </c>
-      <c r="CQ14" s="2" t="inlineStr">
+      <c r="CR14" s="2" t="inlineStr">
         <is>
           <t>JNKSpread</t>
         </is>
       </c>
-      <c r="CR14" s="2" t="inlineStr">
+      <c r="CS14" s="2" t="inlineStr">
         <is>
           <t>StkBonCorr</t>
         </is>
       </c>
-      <c r="CS14" s="2" t="inlineStr">
+      <c r="CT14" s="2" t="inlineStr">
         <is>
           <t>USDGoldRatio</t>
         </is>
       </c>
-      <c r="CT14" s="2" t="inlineStr">
+      <c r="CU14" s="2" t="inlineStr">
         <is>
           <t>SectRotation</t>
         </is>
       </c>
-      <c r="CU14" s="2" t="inlineStr">
+      <c r="CV14" s="2" t="inlineStr">
         <is>
           <t>VIX_TNX_Ratio</t>
         </is>
       </c>
-      <c r="CV14" s="2" t="inlineStr">
+      <c r="CW14" s="2" t="inlineStr">
         <is>
           <t>YldCurveProxy</t>
         </is>
@@ -1178,99 +1171,100 @@
           <t>Volume</t>
         </is>
       </c>
-      <c r="CB15" s="2" t="inlineStr">
-        <is>
-          <t>回报</t>
-        </is>
-      </c>
-      <c r="CC15" s="2" t="n"/>
+      <c r="CB15" s="2" t="n"/>
+      <c r="CC15" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
       <c r="CD15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>High</t>
         </is>
       </c>
       <c r="CE15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="CF15" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="CG15" s="2" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Adj Close</t>
         </is>
       </c>
       <c r="CH15" s="2" t="inlineStr">
         <is>
-          <t>Adj Close</t>
-        </is>
-      </c>
-      <c r="CI15" s="2" t="inlineStr">
-        <is>
           <t>Volume</t>
         </is>
       </c>
+      <c r="CI15" s="2" t="n"/>
       <c r="CJ15" s="2" t="inlineStr">
         <is>
-          <t>回报</t>
-        </is>
-      </c>
-      <c r="CK15" s="2" t="n"/>
+          <t>VIX回报</t>
+        </is>
+      </c>
+      <c r="CK15" s="2" t="inlineStr">
+        <is>
+          <t>VIX_Chg%</t>
+        </is>
+      </c>
       <c r="CL15" s="2" t="inlineStr">
         <is>
-          <t>VIX_close/昨VIX_close-1</t>
+          <t>VIX_5dChg</t>
         </is>
       </c>
       <c r="CM15" s="2" t="inlineStr">
         <is>
-          <t>(TNX_close-昨TNX_close)*100</t>
+          <t>VIX_20dVol</t>
         </is>
       </c>
       <c r="CN15" s="2" t="inlineStr">
         <is>
-          <t>VIX_close/5日前VIX_close-1</t>
+          <t>TNX回报</t>
         </is>
       </c>
       <c r="CO15" s="2" t="inlineStr">
         <is>
-          <t>STDEV(VIX日变化,近20日)</t>
-        </is>
-      </c>
-      <c r="CP15" s="2" t="inlineStr">
+          <t>TNX_ChgBp</t>
+        </is>
+      </c>
+      <c r="CP15" s="2" t="n"/>
+      <c r="CQ15" s="2" t="inlineStr">
         <is>
           <t>HYG-TLT</t>
         </is>
       </c>
-      <c r="CQ15" s="2" t="inlineStr">
+      <c r="CR15" s="2" t="inlineStr">
         <is>
           <t>JNK-TLT</t>
         </is>
       </c>
-      <c r="CR15" s="2" t="inlineStr">
+      <c r="CS15" s="2" t="inlineStr">
         <is>
           <t>CORREL(SPY,TLT,近20日)</t>
         </is>
       </c>
-      <c r="CS15" s="2" t="inlineStr">
+      <c r="CT15" s="2" t="inlineStr">
         <is>
           <t>UUP-GLD</t>
         </is>
       </c>
-      <c r="CT15" s="2" t="inlineStr">
+      <c r="CU15" s="2" t="inlineStr">
         <is>
           <t>XLK-XLF</t>
         </is>
       </c>
-      <c r="CU15" s="2" t="inlineStr">
+      <c r="CV15" s="2" t="inlineStr">
         <is>
           <t>VIX_close/TNX_close</t>
         </is>
       </c>
-      <c r="CV15" s="2" t="inlineStr">
+      <c r="CW15" s="2" t="inlineStr">
         <is>
           <t>TLT-TIP</t>
         </is>
@@ -1399,75 +1393,76 @@
       <c r="CA16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB16" s="4">
-        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC16" s="3" t="n"/>
+      <c r="CB16" s="3" t="n"/>
+      <c r="CC16" s="3" t="n">
+        <v>4.692</v>
+      </c>
       <c r="CD16" s="3" t="n">
-        <v>4.692</v>
+        <v>4.703</v>
       </c>
       <c r="CE16" s="3" t="n">
-        <v>4.703</v>
+        <v>4.668</v>
       </c>
       <c r="CF16" s="3" t="n">
-        <v>4.668</v>
+        <v>4.684</v>
       </c>
       <c r="CG16" s="3" t="n">
         <v>4.684</v>
       </c>
       <c r="CH16" s="3" t="n">
-        <v>4.684</v>
-      </c>
-      <c r="CI16" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI16" s="3" t="n"/>
       <c r="CJ16" s="4">
-        <f>IF(COUNT(CG16:CG17)=2,ROUND((CG16/CG17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK16" s="3" t="n"/>
+        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK16" s="4">
+        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL16" s="4">
-        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM16" s="5">
-        <f>IF(COUNT(CG16:CG17)=2,(CG16-CG17)*100,"")</f>
+        <f>IF(COUNT(BY16:BY21)=6,ROUND((BY16/BY21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM16" s="4">
+        <f>IF(COUNT(CK16:CK35)=20,IFERROR(ROUND(STDEV(CK16:CK35),4),""),"")</f>
         <v/>
       </c>
       <c r="CN16" s="4">
-        <f>IF(COUNT(BY16:BY21)=6,ROUND((BY16/BY21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO16" s="4">
-        <f>IF(COUNT(CL16:CL35)=20,ROUND(STDEV(CL16:CL35),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP16" s="4">
+        <f>IF(COUNT(CF16:CF17)=2,ROUND((CF16/CF17-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO16" s="5">
+        <f>IF(COUNT(CF16:CF17)=2,(CF16-CF17)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP16" s="3" t="n"/>
+      <c r="CQ16" s="4">
         <f>X16-P16</f>
         <v/>
       </c>
-      <c r="CQ16" s="4">
+      <c r="CR16" s="4">
         <f>AF16-P16</f>
         <v/>
       </c>
-      <c r="CR16" s="6">
-        <f>IF(COUNT(H16:H35)=20,CORREL(H16:H35,P16:P35),"")</f>
-        <v/>
-      </c>
-      <c r="CS16" s="4">
+      <c r="CS16" s="6">
+        <f>IF(COUNT(H16:H35)=20,IFERROR(CORREL(H16:H35,P16:P35),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT16" s="4">
         <f>AN16-AV16</f>
         <v/>
       </c>
-      <c r="CT16" s="4">
+      <c r="CU16" s="4">
         <f>BD16-BL16</f>
         <v/>
       </c>
-      <c r="CU16" s="6">
-        <f>BY16/CG16</f>
-        <v/>
-      </c>
-      <c r="CV16" s="4">
+      <c r="CV16" s="6">
+        <f>BY16/CF16</f>
+        <v/>
+      </c>
+      <c r="CW16" s="4">
         <f>P16-BT16</f>
         <v/>
       </c>
@@ -1595,75 +1590,76 @@
       <c r="CA17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB17" s="4">
-        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC17" s="3" t="n"/>
+      <c r="CB17" s="3" t="n"/>
+      <c r="CC17" s="3" t="n">
+        <v>4.662</v>
+      </c>
       <c r="CD17" s="3" t="n">
+        <v>4.703</v>
+      </c>
+      <c r="CE17" s="3" t="n">
         <v>4.662</v>
       </c>
-      <c r="CE17" s="3" t="n">
-        <v>4.703</v>
-      </c>
       <c r="CF17" s="3" t="n">
-        <v>4.662</v>
+        <v>4.699</v>
       </c>
       <c r="CG17" s="3" t="n">
         <v>4.699</v>
       </c>
       <c r="CH17" s="3" t="n">
-        <v>4.699</v>
-      </c>
-      <c r="CI17" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI17" s="3" t="n"/>
       <c r="CJ17" s="4">
-        <f>IF(COUNT(CG17:CG18)=2,ROUND((CG17/CG18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK17" s="3" t="n"/>
+        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK17" s="4">
+        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL17" s="4">
-        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM17" s="5">
-        <f>IF(COUNT(CG17:CG18)=2,(CG17-CG18)*100,"")</f>
+        <f>IF(COUNT(BY17:BY22)=6,ROUND((BY17/BY22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM17" s="4">
+        <f>IF(COUNT(CK17:CK36)=20,IFERROR(ROUND(STDEV(CK17:CK36),4),""),"")</f>
         <v/>
       </c>
       <c r="CN17" s="4">
-        <f>IF(COUNT(BY17:BY22)=6,ROUND((BY17/BY22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO17" s="4">
-        <f>IF(COUNT(CL17:CL36)=20,ROUND(STDEV(CL17:CL36),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP17" s="4">
+        <f>IF(COUNT(CF17:CF18)=2,ROUND((CF17/CF18-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO17" s="5">
+        <f>IF(COUNT(CF17:CF18)=2,(CF17-CF18)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP17" s="3" t="n"/>
+      <c r="CQ17" s="4">
         <f>X17-P17</f>
         <v/>
       </c>
-      <c r="CQ17" s="4">
+      <c r="CR17" s="4">
         <f>AF17-P17</f>
         <v/>
       </c>
-      <c r="CR17" s="6">
-        <f>IF(COUNT(H17:H36)=20,CORREL(H17:H36,P17:P36),"")</f>
-        <v/>
-      </c>
-      <c r="CS17" s="4">
+      <c r="CS17" s="6">
+        <f>IF(COUNT(H17:H36)=20,IFERROR(CORREL(H17:H36,P17:P36),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT17" s="4">
         <f>AN17-AV17</f>
         <v/>
       </c>
-      <c r="CT17" s="4">
+      <c r="CU17" s="4">
         <f>BD17-BL17</f>
         <v/>
       </c>
-      <c r="CU17" s="6">
-        <f>BY17/CG17</f>
-        <v/>
-      </c>
-      <c r="CV17" s="4">
+      <c r="CV17" s="6">
+        <f>BY17/CF17</f>
+        <v/>
+      </c>
+      <c r="CW17" s="4">
         <f>P17-BT17</f>
         <v/>
       </c>
@@ -1899,75 +1895,76 @@
       <c r="CA18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB18" s="4">
-        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC18" s="3" t="n"/>
+      <c r="CB18" s="3" t="n"/>
+      <c r="CC18" s="3" t="n">
+        <v>4.664</v>
+      </c>
       <c r="CD18" s="3" t="n">
-        <v>4.664</v>
+        <v>4.672</v>
       </c>
       <c r="CE18" s="3" t="n">
-        <v>4.672</v>
+        <v>4.603</v>
       </c>
       <c r="CF18" s="3" t="n">
-        <v>4.603</v>
+        <v>4.66</v>
       </c>
       <c r="CG18" s="3" t="n">
         <v>4.66</v>
       </c>
       <c r="CH18" s="3" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="CI18" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI18" s="3" t="n"/>
       <c r="CJ18" s="4">
-        <f>IF(COUNT(CG18:CG19)=2,ROUND((CG18/CG19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK18" s="3" t="n"/>
+        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK18" s="4">
+        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL18" s="4">
-        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM18" s="5">
-        <f>IF(COUNT(CG18:CG19)=2,(CG18-CG19)*100,"")</f>
+        <f>IF(COUNT(BY18:BY23)=6,ROUND((BY18/BY23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM18" s="4">
+        <f>IF(COUNT(CK18:CK37)=20,IFERROR(ROUND(STDEV(CK18:CK37),4),""),"")</f>
         <v/>
       </c>
       <c r="CN18" s="4">
-        <f>IF(COUNT(BY18:BY23)=6,ROUND((BY18/BY23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO18" s="4">
-        <f>IF(COUNT(CL18:CL37)=20,ROUND(STDEV(CL18:CL37),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP18" s="4">
+        <f>IF(COUNT(CF18:CF19)=2,ROUND((CF18/CF19-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO18" s="5">
+        <f>IF(COUNT(CF18:CF19)=2,(CF18-CF19)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP18" s="3" t="n"/>
+      <c r="CQ18" s="4">
         <f>X18-P18</f>
         <v/>
       </c>
-      <c r="CQ18" s="4">
+      <c r="CR18" s="4">
         <f>AF18-P18</f>
         <v/>
       </c>
-      <c r="CR18" s="6">
-        <f>IF(COUNT(H18:H37)=20,CORREL(H18:H37,P18:P37),"")</f>
-        <v/>
-      </c>
-      <c r="CS18" s="4">
+      <c r="CS18" s="6">
+        <f>IF(COUNT(H18:H37)=20,IFERROR(CORREL(H18:H37,P18:P37),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT18" s="4">
         <f>AN18-AV18</f>
         <v/>
       </c>
-      <c r="CT18" s="4">
+      <c r="CU18" s="4">
         <f>BD18-BL18</f>
         <v/>
       </c>
-      <c r="CU18" s="6">
-        <f>BY18/CG18</f>
-        <v/>
-      </c>
-      <c r="CV18" s="4">
+      <c r="CV18" s="6">
+        <f>BY18/CF18</f>
+        <v/>
+      </c>
+      <c r="CW18" s="4">
         <f>P18-BT18</f>
         <v/>
       </c>
@@ -2203,75 +2200,76 @@
       <c r="CA19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB19" s="4">
-        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC19" s="3" t="n"/>
+      <c r="CB19" s="3" t="n"/>
+      <c r="CC19" s="3" t="n">
+        <v>4.643</v>
+      </c>
       <c r="CD19" s="3" t="n">
-        <v>4.643</v>
+        <v>4.676</v>
       </c>
       <c r="CE19" s="3" t="n">
-        <v>4.676</v>
+        <v>4.635</v>
       </c>
       <c r="CF19" s="3" t="n">
-        <v>4.635</v>
+        <v>4.67</v>
       </c>
       <c r="CG19" s="3" t="n">
         <v>4.67</v>
       </c>
       <c r="CH19" s="3" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="CI19" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI19" s="3" t="n"/>
       <c r="CJ19" s="4">
-        <f>IF(COUNT(CG19:CG20)=2,ROUND((CG19/CG20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK19" s="3" t="n"/>
+        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK19" s="4">
+        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL19" s="4">
-        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM19" s="5">
-        <f>IF(COUNT(CG19:CG20)=2,(CG19-CG20)*100,"")</f>
+        <f>IF(COUNT(BY19:BY24)=6,ROUND((BY19/BY24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM19" s="4">
+        <f>IF(COUNT(CK19:CK38)=20,IFERROR(ROUND(STDEV(CK19:CK38),4),""),"")</f>
         <v/>
       </c>
       <c r="CN19" s="4">
-        <f>IF(COUNT(BY19:BY24)=6,ROUND((BY19/BY24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO19" s="4">
-        <f>IF(COUNT(CL19:CL38)=20,ROUND(STDEV(CL19:CL38),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP19" s="4">
+        <f>IF(COUNT(CF19:CF20)=2,ROUND((CF19/CF20-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO19" s="5">
+        <f>IF(COUNT(CF19:CF20)=2,(CF19-CF20)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP19" s="3" t="n"/>
+      <c r="CQ19" s="4">
         <f>X19-P19</f>
         <v/>
       </c>
-      <c r="CQ19" s="4">
+      <c r="CR19" s="4">
         <f>AF19-P19</f>
         <v/>
       </c>
-      <c r="CR19" s="6">
-        <f>IF(COUNT(H19:H38)=20,CORREL(H19:H38,P19:P38),"")</f>
-        <v/>
-      </c>
-      <c r="CS19" s="4">
+      <c r="CS19" s="6">
+        <f>IF(COUNT(H19:H38)=20,IFERROR(CORREL(H19:H38,P19:P38),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT19" s="4">
         <f>AN19-AV19</f>
         <v/>
       </c>
-      <c r="CT19" s="4">
+      <c r="CU19" s="4">
         <f>BD19-BL19</f>
         <v/>
       </c>
-      <c r="CU19" s="6">
-        <f>BY19/CG19</f>
-        <v/>
-      </c>
-      <c r="CV19" s="4">
+      <c r="CV19" s="6">
+        <f>BY19/CF19</f>
+        <v/>
+      </c>
+      <c r="CW19" s="4">
         <f>P19-BT19</f>
         <v/>
       </c>
@@ -2507,75 +2505,76 @@
       <c r="CA20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB20" s="4">
-        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC20" s="3" t="n"/>
+      <c r="CB20" s="3" t="n"/>
+      <c r="CC20" s="3" t="n">
+        <v>4.609</v>
+      </c>
       <c r="CD20" s="3" t="n">
-        <v>4.609</v>
+        <v>4.639</v>
       </c>
       <c r="CE20" s="3" t="n">
-        <v>4.639</v>
+        <v>4.607</v>
       </c>
       <c r="CF20" s="3" t="n">
-        <v>4.607</v>
+        <v>4.617</v>
       </c>
       <c r="CG20" s="3" t="n">
         <v>4.617</v>
       </c>
       <c r="CH20" s="3" t="n">
-        <v>4.617</v>
-      </c>
-      <c r="CI20" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI20" s="3" t="n"/>
       <c r="CJ20" s="4">
-        <f>IF(COUNT(CG20:CG21)=2,ROUND((CG20/CG21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK20" s="3" t="n"/>
+        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK20" s="4">
+        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL20" s="4">
-        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM20" s="5">
-        <f>IF(COUNT(CG20:CG21)=2,(CG20-CG21)*100,"")</f>
+        <f>IF(COUNT(BY20:BY25)=6,ROUND((BY20/BY25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM20" s="4">
+        <f>IF(COUNT(CK20:CK39)=20,IFERROR(ROUND(STDEV(CK20:CK39),4),""),"")</f>
         <v/>
       </c>
       <c r="CN20" s="4">
-        <f>IF(COUNT(BY20:BY25)=6,ROUND((BY20/BY25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO20" s="4">
-        <f>IF(COUNT(CL20:CL39)=20,ROUND(STDEV(CL20:CL39),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP20" s="4">
+        <f>IF(COUNT(CF20:CF21)=2,ROUND((CF20/CF21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO20" s="5">
+        <f>IF(COUNT(CF20:CF21)=2,(CF20-CF21)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP20" s="3" t="n"/>
+      <c r="CQ20" s="4">
         <f>X20-P20</f>
         <v/>
       </c>
-      <c r="CQ20" s="4">
+      <c r="CR20" s="4">
         <f>AF20-P20</f>
         <v/>
       </c>
-      <c r="CR20" s="6">
-        <f>IF(COUNT(H20:H39)=20,CORREL(H20:H39,P20:P39),"")</f>
-        <v/>
-      </c>
-      <c r="CS20" s="4">
+      <c r="CS20" s="6">
+        <f>IF(COUNT(H20:H39)=20,IFERROR(CORREL(H20:H39,P20:P39),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT20" s="4">
         <f>AN20-AV20</f>
         <v/>
       </c>
-      <c r="CT20" s="4">
+      <c r="CU20" s="4">
         <f>BD20-BL20</f>
         <v/>
       </c>
-      <c r="CU20" s="6">
-        <f>BY20/CG20</f>
-        <v/>
-      </c>
-      <c r="CV20" s="4">
+      <c r="CV20" s="6">
+        <f>BY20/CF20</f>
+        <v/>
+      </c>
+      <c r="CW20" s="4">
         <f>P20-BT20</f>
         <v/>
       </c>
@@ -2811,75 +2810,76 @@
       <c r="CA21" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB21" s="4">
-        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC21" s="3" t="n"/>
+      <c r="CB21" s="3" t="n"/>
+      <c r="CC21" s="3" t="n">
+        <v>4.665</v>
+      </c>
       <c r="CD21" s="3" t="n">
-        <v>4.665</v>
+        <v>4.668</v>
       </c>
       <c r="CE21" s="3" t="n">
-        <v>4.668</v>
+        <v>4.619</v>
       </c>
       <c r="CF21" s="3" t="n">
-        <v>4.619</v>
+        <v>4.627</v>
       </c>
       <c r="CG21" s="3" t="n">
         <v>4.627</v>
       </c>
       <c r="CH21" s="3" t="n">
-        <v>4.627</v>
-      </c>
-      <c r="CI21" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI21" s="3" t="n"/>
       <c r="CJ21" s="4">
-        <f>IF(COUNT(CG21:CG22)=2,ROUND((CG21/CG22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK21" s="3" t="n"/>
+        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK21" s="4">
+        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL21" s="4">
-        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM21" s="5">
-        <f>IF(COUNT(CG21:CG22)=2,(CG21-CG22)*100,"")</f>
+        <f>IF(COUNT(BY21:BY26)=6,ROUND((BY21/BY26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM21" s="4">
+        <f>IF(COUNT(CK21:CK40)=20,IFERROR(ROUND(STDEV(CK21:CK40),4),""),"")</f>
         <v/>
       </c>
       <c r="CN21" s="4">
-        <f>IF(COUNT(BY21:BY26)=6,ROUND((BY21/BY26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO21" s="4">
-        <f>IF(COUNT(CL21:CL40)=20,ROUND(STDEV(CL21:CL40),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP21" s="4">
+        <f>IF(COUNT(CF21:CF22)=2,ROUND((CF21/CF22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO21" s="5">
+        <f>IF(COUNT(CF21:CF22)=2,(CF21-CF22)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP21" s="3" t="n"/>
+      <c r="CQ21" s="4">
         <f>X21-P21</f>
         <v/>
       </c>
-      <c r="CQ21" s="4">
+      <c r="CR21" s="4">
         <f>AF21-P21</f>
         <v/>
       </c>
-      <c r="CR21" s="6">
-        <f>IF(COUNT(H21:H40)=20,CORREL(H21:H40,P21:P40),"")</f>
-        <v/>
-      </c>
-      <c r="CS21" s="4">
+      <c r="CS21" s="6">
+        <f>IF(COUNT(H21:H40)=20,IFERROR(CORREL(H21:H40,P21:P40),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT21" s="4">
         <f>AN21-AV21</f>
         <v/>
       </c>
-      <c r="CT21" s="4">
+      <c r="CU21" s="4">
         <f>BD21-BL21</f>
         <v/>
       </c>
-      <c r="CU21" s="6">
-        <f>BY21/CG21</f>
-        <v/>
-      </c>
-      <c r="CV21" s="4">
+      <c r="CV21" s="6">
+        <f>BY21/CF21</f>
+        <v/>
+      </c>
+      <c r="CW21" s="4">
         <f>P21-BT21</f>
         <v/>
       </c>
@@ -3115,75 +3115,76 @@
       <c r="CA22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB22" s="4">
-        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC22" s="3" t="n"/>
+      <c r="CB22" s="3" t="n"/>
+      <c r="CC22" s="3" t="n">
+        <v>4.671</v>
+      </c>
       <c r="CD22" s="3" t="n">
+        <v>4.702</v>
+      </c>
+      <c r="CE22" s="3" t="n">
         <v>4.671</v>
       </c>
-      <c r="CE22" s="3" t="n">
-        <v>4.702</v>
-      </c>
       <c r="CF22" s="3" t="n">
-        <v>4.671</v>
+        <v>4.686</v>
       </c>
       <c r="CG22" s="3" t="n">
         <v>4.686</v>
       </c>
       <c r="CH22" s="3" t="n">
-        <v>4.686</v>
-      </c>
-      <c r="CI22" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI22" s="3" t="n"/>
       <c r="CJ22" s="4">
-        <f>IF(COUNT(CG22:CG23)=2,ROUND((CG22/CG23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK22" s="3" t="n"/>
+        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK22" s="4">
+        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL22" s="4">
-        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM22" s="5">
-        <f>IF(COUNT(CG22:CG23)=2,(CG22-CG23)*100,"")</f>
+        <f>IF(COUNT(BY22:BY27)=6,ROUND((BY22/BY27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM22" s="4">
+        <f>IF(COUNT(CK22:CK41)=20,IFERROR(ROUND(STDEV(CK22:CK41),4),""),"")</f>
         <v/>
       </c>
       <c r="CN22" s="4">
-        <f>IF(COUNT(BY22:BY27)=6,ROUND((BY22/BY27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO22" s="4">
-        <f>IF(COUNT(CL22:CL41)=20,ROUND(STDEV(CL22:CL41),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP22" s="4">
+        <f>IF(COUNT(CF22:CF23)=2,ROUND((CF22/CF23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO22" s="5">
+        <f>IF(COUNT(CF22:CF23)=2,(CF22-CF23)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP22" s="3" t="n"/>
+      <c r="CQ22" s="4">
         <f>X22-P22</f>
         <v/>
       </c>
-      <c r="CQ22" s="4">
+      <c r="CR22" s="4">
         <f>AF22-P22</f>
         <v/>
       </c>
-      <c r="CR22" s="6">
-        <f>IF(COUNT(H22:H41)=20,CORREL(H22:H41,P22:P41),"")</f>
-        <v/>
-      </c>
-      <c r="CS22" s="4">
+      <c r="CS22" s="6">
+        <f>IF(COUNT(H22:H41)=20,IFERROR(CORREL(H22:H41,P22:P41),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT22" s="4">
         <f>AN22-AV22</f>
         <v/>
       </c>
-      <c r="CT22" s="4">
+      <c r="CU22" s="4">
         <f>BD22-BL22</f>
         <v/>
       </c>
-      <c r="CU22" s="6">
-        <f>BY22/CG22</f>
-        <v/>
-      </c>
-      <c r="CV22" s="4">
+      <c r="CV22" s="6">
+        <f>BY22/CF22</f>
+        <v/>
+      </c>
+      <c r="CW22" s="4">
         <f>P22-BT22</f>
         <v/>
       </c>
@@ -3419,75 +3420,76 @@
       <c r="CA23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB23" s="4">
-        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC23" s="3" t="n"/>
+      <c r="CB23" s="3" t="n"/>
+      <c r="CC23" s="3" t="n">
+        <v>4.684</v>
+      </c>
       <c r="CD23" s="3" t="n">
-        <v>4.684</v>
+        <v>4.747</v>
       </c>
       <c r="CE23" s="3" t="n">
-        <v>4.747</v>
+        <v>4.682</v>
       </c>
       <c r="CF23" s="3" t="n">
-        <v>4.682</v>
+        <v>4.745</v>
       </c>
       <c r="CG23" s="3" t="n">
         <v>4.745</v>
       </c>
       <c r="CH23" s="3" t="n">
-        <v>4.745</v>
-      </c>
-      <c r="CI23" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI23" s="3" t="n"/>
       <c r="CJ23" s="4">
-        <f>IF(COUNT(CG23:CG24)=2,ROUND((CG23/CG24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK23" s="3" t="n"/>
+        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK23" s="4">
+        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL23" s="4">
-        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM23" s="5">
-        <f>IF(COUNT(CG23:CG24)=2,(CG23-CG24)*100,"")</f>
+        <f>IF(COUNT(BY23:BY28)=6,ROUND((BY23/BY28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM23" s="4">
+        <f>IF(COUNT(CK23:CK42)=20,IFERROR(ROUND(STDEV(CK23:CK42),4),""),"")</f>
         <v/>
       </c>
       <c r="CN23" s="4">
-        <f>IF(COUNT(BY23:BY28)=6,ROUND((BY23/BY28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO23" s="4">
-        <f>IF(COUNT(CL23:CL42)=20,ROUND(STDEV(CL23:CL42),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP23" s="4">
+        <f>IF(COUNT(CF23:CF24)=2,ROUND((CF23/CF24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO23" s="5">
+        <f>IF(COUNT(CF23:CF24)=2,(CF23-CF24)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP23" s="3" t="n"/>
+      <c r="CQ23" s="4">
         <f>X23-P23</f>
         <v/>
       </c>
-      <c r="CQ23" s="4">
+      <c r="CR23" s="4">
         <f>AF23-P23</f>
         <v/>
       </c>
-      <c r="CR23" s="6">
-        <f>IF(COUNT(H23:H42)=20,CORREL(H23:H42,P23:P42),"")</f>
-        <v/>
-      </c>
-      <c r="CS23" s="4">
+      <c r="CS23" s="6">
+        <f>IF(COUNT(H23:H42)=20,IFERROR(CORREL(H23:H42,P23:P42),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT23" s="4">
         <f>AN23-AV23</f>
         <v/>
       </c>
-      <c r="CT23" s="4">
+      <c r="CU23" s="4">
         <f>BD23-BL23</f>
         <v/>
       </c>
-      <c r="CU23" s="6">
-        <f>BY23/CG23</f>
-        <v/>
-      </c>
-      <c r="CV23" s="4">
+      <c r="CV23" s="6">
+        <f>BY23/CF23</f>
+        <v/>
+      </c>
+      <c r="CW23" s="4">
         <f>P23-BT23</f>
         <v/>
       </c>
@@ -3723,75 +3725,76 @@
       <c r="CA24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB24" s="4">
-        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC24" s="3" t="n"/>
+      <c r="CB24" s="3" t="n"/>
+      <c r="CC24" s="3" t="n">
+        <v>4.669</v>
+      </c>
       <c r="CD24" s="3" t="n">
-        <v>4.669</v>
+        <v>4.686</v>
       </c>
       <c r="CE24" s="3" t="n">
-        <v>4.686</v>
+        <v>4.651</v>
       </c>
       <c r="CF24" s="3" t="n">
-        <v>4.651</v>
+        <v>4.663</v>
       </c>
       <c r="CG24" s="3" t="n">
         <v>4.663</v>
       </c>
       <c r="CH24" s="3" t="n">
-        <v>4.663</v>
-      </c>
-      <c r="CI24" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI24" s="3" t="n"/>
       <c r="CJ24" s="4">
-        <f>IF(COUNT(CG24:CG25)=2,ROUND((CG24/CG25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK24" s="3" t="n"/>
+        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK24" s="4">
+        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL24" s="4">
-        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM24" s="5">
-        <f>IF(COUNT(CG24:CG25)=2,(CG24-CG25)*100,"")</f>
+        <f>IF(COUNT(BY24:BY29)=6,ROUND((BY24/BY29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM24" s="4">
+        <f>IF(COUNT(CK24:CK43)=20,IFERROR(ROUND(STDEV(CK24:CK43),4),""),"")</f>
         <v/>
       </c>
       <c r="CN24" s="4">
-        <f>IF(COUNT(BY24:BY29)=6,ROUND((BY24/BY29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO24" s="4">
-        <f>IF(COUNT(CL24:CL43)=20,ROUND(STDEV(CL24:CL43),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP24" s="4">
+        <f>IF(COUNT(CF24:CF25)=2,ROUND((CF24/CF25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO24" s="5">
+        <f>IF(COUNT(CF24:CF25)=2,(CF24-CF25)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP24" s="3" t="n"/>
+      <c r="CQ24" s="4">
         <f>X24-P24</f>
         <v/>
       </c>
-      <c r="CQ24" s="4">
+      <c r="CR24" s="4">
         <f>AF24-P24</f>
         <v/>
       </c>
-      <c r="CR24" s="6">
-        <f>IF(COUNT(H24:H43)=20,CORREL(H24:H43,P24:P43),"")</f>
-        <v/>
-      </c>
-      <c r="CS24" s="4">
+      <c r="CS24" s="6">
+        <f>IF(COUNT(H24:H43)=20,IFERROR(CORREL(H24:H43,P24:P43),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT24" s="4">
         <f>AN24-AV24</f>
         <v/>
       </c>
-      <c r="CT24" s="4">
+      <c r="CU24" s="4">
         <f>BD24-BL24</f>
         <v/>
       </c>
-      <c r="CU24" s="6">
-        <f>BY24/CG24</f>
-        <v/>
-      </c>
-      <c r="CV24" s="4">
+      <c r="CV24" s="6">
+        <f>BY24/CF24</f>
+        <v/>
+      </c>
+      <c r="CW24" s="4">
         <f>P24-BT24</f>
         <v/>
       </c>
@@ -4027,75 +4030,76 @@
       <c r="CA25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB25" s="4">
-        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC25" s="3" t="n"/>
+      <c r="CB25" s="3" t="n"/>
+      <c r="CC25" s="3" t="n">
+        <v>4.637</v>
+      </c>
       <c r="CD25" s="3" t="n">
-        <v>4.637</v>
+        <v>4.655</v>
       </c>
       <c r="CE25" s="3" t="n">
-        <v>4.655</v>
+        <v>4.61</v>
       </c>
       <c r="CF25" s="3" t="n">
-        <v>4.61</v>
+        <v>4.622</v>
       </c>
       <c r="CG25" s="3" t="n">
         <v>4.622</v>
       </c>
       <c r="CH25" s="3" t="n">
-        <v>4.622</v>
-      </c>
-      <c r="CI25" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI25" s="3" t="n"/>
       <c r="CJ25" s="4">
-        <f>IF(COUNT(CG25:CG26)=2,ROUND((CG25/CG26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK25" s="3" t="n"/>
+        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK25" s="4">
+        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL25" s="4">
-        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM25" s="5">
-        <f>IF(COUNT(CG25:CG26)=2,(CG25-CG26)*100,"")</f>
+        <f>IF(COUNT(BY25:BY30)=6,ROUND((BY25/BY30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM25" s="4">
+        <f>IF(COUNT(CK25:CK44)=20,IFERROR(ROUND(STDEV(CK25:CK44),4),""),"")</f>
         <v/>
       </c>
       <c r="CN25" s="4">
-        <f>IF(COUNT(BY25:BY30)=6,ROUND((BY25/BY30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO25" s="4">
-        <f>IF(COUNT(CL25:CL44)=20,ROUND(STDEV(CL25:CL44),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP25" s="4">
+        <f>IF(COUNT(CF25:CF26)=2,ROUND((CF25/CF26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO25" s="5">
+        <f>IF(COUNT(CF25:CF26)=2,(CF25-CF26)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP25" s="3" t="n"/>
+      <c r="CQ25" s="4">
         <f>X25-P25</f>
         <v/>
       </c>
-      <c r="CQ25" s="4">
+      <c r="CR25" s="4">
         <f>AF25-P25</f>
         <v/>
       </c>
-      <c r="CR25" s="6">
-        <f>IF(COUNT(H25:H44)=20,CORREL(H25:H44,P25:P44),"")</f>
-        <v/>
-      </c>
-      <c r="CS25" s="4">
+      <c r="CS25" s="6">
+        <f>IF(COUNT(H25:H44)=20,IFERROR(CORREL(H25:H44,P25:P44),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT25" s="4">
         <f>AN25-AV25</f>
         <v/>
       </c>
-      <c r="CT25" s="4">
+      <c r="CU25" s="4">
         <f>BD25-BL25</f>
         <v/>
       </c>
-      <c r="CU25" s="6">
-        <f>BY25/CG25</f>
-        <v/>
-      </c>
-      <c r="CV25" s="4">
+      <c r="CV25" s="6">
+        <f>BY25/CF25</f>
+        <v/>
+      </c>
+      <c r="CW25" s="4">
         <f>P25-BT25</f>
         <v/>
       </c>
@@ -4331,75 +4335,76 @@
       <c r="CA26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB26" s="4">
-        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC26" s="3" t="n"/>
+      <c r="CB26" s="3" t="n"/>
+      <c r="CC26" s="3" t="n">
+        <v>4.63</v>
+      </c>
       <c r="CD26" s="3" t="n">
-        <v>4.63</v>
+        <v>4.635</v>
       </c>
       <c r="CE26" s="3" t="n">
-        <v>4.635</v>
+        <v>4.588</v>
       </c>
       <c r="CF26" s="3" t="n">
-        <v>4.588</v>
+        <v>4.604</v>
       </c>
       <c r="CG26" s="3" t="n">
         <v>4.604</v>
       </c>
       <c r="CH26" s="3" t="n">
-        <v>4.604</v>
-      </c>
-      <c r="CI26" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI26" s="3" t="n"/>
       <c r="CJ26" s="4">
-        <f>IF(COUNT(CG26:CG27)=2,ROUND((CG26/CG27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK26" s="3" t="n"/>
+        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK26" s="4">
+        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL26" s="4">
-        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM26" s="5">
-        <f>IF(COUNT(CG26:CG27)=2,(CG26-CG27)*100,"")</f>
+        <f>IF(COUNT(BY26:BY31)=6,ROUND((BY26/BY31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM26" s="4">
+        <f>IF(COUNT(CK26:CK45)=20,IFERROR(ROUND(STDEV(CK26:CK45),4),""),"")</f>
         <v/>
       </c>
       <c r="CN26" s="4">
-        <f>IF(COUNT(BY26:BY31)=6,ROUND((BY26/BY31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO26" s="4">
-        <f>IF(COUNT(CL26:CL45)=20,ROUND(STDEV(CL26:CL45),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP26" s="4">
+        <f>IF(COUNT(CF26:CF27)=2,ROUND((CF26/CF27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO26" s="5">
+        <f>IF(COUNT(CF26:CF27)=2,(CF26-CF27)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP26" s="3" t="n"/>
+      <c r="CQ26" s="4">
         <f>X26-P26</f>
         <v/>
       </c>
-      <c r="CQ26" s="4">
+      <c r="CR26" s="4">
         <f>AF26-P26</f>
         <v/>
       </c>
-      <c r="CR26" s="6">
-        <f>IF(COUNT(H26:H45)=20,CORREL(H26:H45,P26:P45),"")</f>
-        <v/>
-      </c>
-      <c r="CS26" s="4">
+      <c r="CS26" s="6">
+        <f>IF(COUNT(H26:H45)=20,IFERROR(CORREL(H26:H45,P26:P45),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT26" s="4">
         <f>AN26-AV26</f>
         <v/>
       </c>
-      <c r="CT26" s="4">
+      <c r="CU26" s="4">
         <f>BD26-BL26</f>
         <v/>
       </c>
-      <c r="CU26" s="6">
-        <f>BY26/CG26</f>
-        <v/>
-      </c>
-      <c r="CV26" s="4">
+      <c r="CV26" s="6">
+        <f>BY26/CF26</f>
+        <v/>
+      </c>
+      <c r="CW26" s="4">
         <f>P26-BT26</f>
         <v/>
       </c>
@@ -4635,75 +4640,76 @@
       <c r="CA27" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB27" s="4">
-        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC27" s="3" t="n"/>
+      <c r="CB27" s="3" t="n"/>
+      <c r="CC27" s="3" t="n">
+        <v>4.647</v>
+      </c>
       <c r="CD27" s="3" t="n">
-        <v>4.647</v>
+        <v>4.665</v>
       </c>
       <c r="CE27" s="3" t="n">
-        <v>4.665</v>
+        <v>4.63</v>
       </c>
       <c r="CF27" s="3" t="n">
-        <v>4.63</v>
+        <v>4.641</v>
       </c>
       <c r="CG27" s="3" t="n">
         <v>4.641</v>
       </c>
       <c r="CH27" s="3" t="n">
-        <v>4.641</v>
-      </c>
-      <c r="CI27" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI27" s="3" t="n"/>
       <c r="CJ27" s="4">
-        <f>IF(COUNT(CG27:CG28)=2,ROUND((CG27/CG28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK27" s="3" t="n"/>
+        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK27" s="4">
+        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL27" s="4">
-        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM27" s="5">
-        <f>IF(COUNT(CG27:CG28)=2,(CG27-CG28)*100,"")</f>
+        <f>IF(COUNT(BY27:BY32)=6,ROUND((BY27/BY32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM27" s="4">
+        <f>IF(COUNT(CK27:CK46)=20,IFERROR(ROUND(STDEV(CK27:CK46),4),""),"")</f>
         <v/>
       </c>
       <c r="CN27" s="4">
-        <f>IF(COUNT(BY27:BY32)=6,ROUND((BY27/BY32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO27" s="4">
-        <f>IF(COUNT(CL27:CL46)=20,ROUND(STDEV(CL27:CL46),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP27" s="4">
+        <f>IF(COUNT(CF27:CF28)=2,ROUND((CF27/CF28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO27" s="5">
+        <f>IF(COUNT(CF27:CF28)=2,(CF27-CF28)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP27" s="3" t="n"/>
+      <c r="CQ27" s="4">
         <f>X27-P27</f>
         <v/>
       </c>
-      <c r="CQ27" s="4">
+      <c r="CR27" s="4">
         <f>AF27-P27</f>
         <v/>
       </c>
-      <c r="CR27" s="6">
-        <f>IF(COUNT(H27:H46)=20,CORREL(H27:H46,P27:P46),"")</f>
-        <v/>
-      </c>
-      <c r="CS27" s="4">
+      <c r="CS27" s="6">
+        <f>IF(COUNT(H27:H46)=20,IFERROR(CORREL(H27:H46,P27:P46),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT27" s="4">
         <f>AN27-AV27</f>
         <v/>
       </c>
-      <c r="CT27" s="4">
+      <c r="CU27" s="4">
         <f>BD27-BL27</f>
         <v/>
       </c>
-      <c r="CU27" s="6">
-        <f>BY27/CG27</f>
-        <v/>
-      </c>
-      <c r="CV27" s="4">
+      <c r="CV27" s="6">
+        <f>BY27/CF27</f>
+        <v/>
+      </c>
+      <c r="CW27" s="4">
         <f>P27-BT27</f>
         <v/>
       </c>
@@ -4939,75 +4945,76 @@
       <c r="CA28" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB28" s="4">
-        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC28" s="3" t="n"/>
+      <c r="CB28" s="3" t="n"/>
+      <c r="CC28" s="3" t="n">
+        <v>4.683</v>
+      </c>
       <c r="CD28" s="3" t="n">
-        <v>4.683</v>
+        <v>4.691</v>
       </c>
       <c r="CE28" s="3" t="n">
-        <v>4.691</v>
+        <v>4.651</v>
       </c>
       <c r="CF28" s="3" t="n">
-        <v>4.651</v>
+        <v>4.679</v>
       </c>
       <c r="CG28" s="3" t="n">
         <v>4.679</v>
       </c>
       <c r="CH28" s="3" t="n">
-        <v>4.679</v>
-      </c>
-      <c r="CI28" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI28" s="3" t="n"/>
       <c r="CJ28" s="4">
-        <f>IF(COUNT(CG28:CG29)=2,ROUND((CG28/CG29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK28" s="3" t="n"/>
+        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK28" s="4">
+        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL28" s="4">
-        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM28" s="5">
-        <f>IF(COUNT(CG28:CG29)=2,(CG28-CG29)*100,"")</f>
+        <f>IF(COUNT(BY28:BY33)=6,ROUND((BY28/BY33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM28" s="4">
+        <f>IF(COUNT(CK28:CK47)=20,IFERROR(ROUND(STDEV(CK28:CK47),4),""),"")</f>
         <v/>
       </c>
       <c r="CN28" s="4">
-        <f>IF(COUNT(BY28:BY33)=6,ROUND((BY28/BY33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO28" s="4">
-        <f>IF(COUNT(CL28:CL47)=20,ROUND(STDEV(CL28:CL47),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP28" s="4">
+        <f>IF(COUNT(CF28:CF29)=2,ROUND((CF28/CF29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO28" s="5">
+        <f>IF(COUNT(CF28:CF29)=2,(CF28-CF29)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP28" s="3" t="n"/>
+      <c r="CQ28" s="4">
         <f>X28-P28</f>
         <v/>
       </c>
-      <c r="CQ28" s="4">
+      <c r="CR28" s="4">
         <f>AF28-P28</f>
         <v/>
       </c>
-      <c r="CR28" s="6">
-        <f>IF(COUNT(H28:H47)=20,CORREL(H28:H47,P28:P47),"")</f>
-        <v/>
-      </c>
-      <c r="CS28" s="4">
+      <c r="CS28" s="6">
+        <f>IF(COUNT(H28:H47)=20,IFERROR(CORREL(H28:H47,P28:P47),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT28" s="4">
         <f>AN28-AV28</f>
         <v/>
       </c>
-      <c r="CT28" s="4">
+      <c r="CU28" s="4">
         <f>BD28-BL28</f>
         <v/>
       </c>
-      <c r="CU28" s="6">
-        <f>BY28/CG28</f>
-        <v/>
-      </c>
-      <c r="CV28" s="4">
+      <c r="CV28" s="6">
+        <f>BY28/CF28</f>
+        <v/>
+      </c>
+      <c r="CW28" s="4">
         <f>P28-BT28</f>
         <v/>
       </c>
@@ -5243,75 +5250,76 @@
       <c r="CA29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB29" s="4">
-        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC29" s="3" t="n"/>
+      <c r="CB29" s="3" t="n"/>
+      <c r="CC29" s="3" t="n">
+        <v>4.699</v>
+      </c>
       <c r="CD29" s="3" t="n">
-        <v>4.699</v>
+        <v>4.714</v>
       </c>
       <c r="CE29" s="3" t="n">
-        <v>4.714</v>
+        <v>4.693</v>
       </c>
       <c r="CF29" s="3" t="n">
-        <v>4.693</v>
+        <v>4.703</v>
       </c>
       <c r="CG29" s="3" t="n">
         <v>4.703</v>
       </c>
       <c r="CH29" s="3" t="n">
-        <v>4.703</v>
-      </c>
-      <c r="CI29" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI29" s="3" t="n"/>
       <c r="CJ29" s="4">
-        <f>IF(COUNT(CG29:CG30)=2,ROUND((CG29/CG30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK29" s="3" t="n"/>
+        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK29" s="4">
+        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL29" s="4">
-        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM29" s="5">
-        <f>IF(COUNT(CG29:CG30)=2,(CG29-CG30)*100,"")</f>
+        <f>IF(COUNT(BY29:BY34)=6,ROUND((BY29/BY34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM29" s="4">
+        <f>IF(COUNT(CK29:CK48)=20,IFERROR(ROUND(STDEV(CK29:CK48),4),""),"")</f>
         <v/>
       </c>
       <c r="CN29" s="4">
-        <f>IF(COUNT(BY29:BY34)=6,ROUND((BY29/BY34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO29" s="4">
-        <f>IF(COUNT(CL29:CL48)=20,ROUND(STDEV(CL29:CL48),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP29" s="4">
+        <f>IF(COUNT(CF29:CF30)=2,ROUND((CF29/CF30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO29" s="5">
+        <f>IF(COUNT(CF29:CF30)=2,(CF29-CF30)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP29" s="3" t="n"/>
+      <c r="CQ29" s="4">
         <f>X29-P29</f>
         <v/>
       </c>
-      <c r="CQ29" s="4">
+      <c r="CR29" s="4">
         <f>AF29-P29</f>
         <v/>
       </c>
-      <c r="CR29" s="6">
-        <f>IF(COUNT(H29:H48)=20,CORREL(H29:H48,P29:P48),"")</f>
-        <v/>
-      </c>
-      <c r="CS29" s="4">
+      <c r="CS29" s="6">
+        <f>IF(COUNT(H29:H48)=20,IFERROR(CORREL(H29:H48,P29:P48),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT29" s="4">
         <f>AN29-AV29</f>
         <v/>
       </c>
-      <c r="CT29" s="4">
+      <c r="CU29" s="4">
         <f>BD29-BL29</f>
         <v/>
       </c>
-      <c r="CU29" s="6">
-        <f>BY29/CG29</f>
-        <v/>
-      </c>
-      <c r="CV29" s="4">
+      <c r="CV29" s="6">
+        <f>BY29/CF29</f>
+        <v/>
+      </c>
+      <c r="CW29" s="4">
         <f>P29-BT29</f>
         <v/>
       </c>
@@ -5547,75 +5555,76 @@
       <c r="CA30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB30" s="4">
-        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC30" s="3" t="n"/>
+      <c r="CB30" s="3" t="n"/>
+      <c r="CC30" s="3" t="n">
+        <v>4.64</v>
+      </c>
       <c r="CD30" s="3" t="n">
-        <v>4.64</v>
+        <v>4.661</v>
       </c>
       <c r="CE30" s="3" t="n">
-        <v>4.661</v>
+        <v>4.632</v>
       </c>
       <c r="CF30" s="3" t="n">
-        <v>4.632</v>
+        <v>4.657</v>
       </c>
       <c r="CG30" s="3" t="n">
         <v>4.657</v>
       </c>
       <c r="CH30" s="3" t="n">
-        <v>4.657</v>
-      </c>
-      <c r="CI30" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI30" s="3" t="n"/>
       <c r="CJ30" s="4">
-        <f>IF(COUNT(CG30:CG31)=2,ROUND((CG30/CG31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK30" s="3" t="n"/>
+        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK30" s="4">
+        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL30" s="4">
-        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM30" s="5">
-        <f>IF(COUNT(CG30:CG31)=2,(CG30-CG31)*100,"")</f>
+        <f>IF(COUNT(BY30:BY35)=6,ROUND((BY30/BY35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM30" s="4">
+        <f>IF(COUNT(CK30:CK49)=20,IFERROR(ROUND(STDEV(CK30:CK49),4),""),"")</f>
         <v/>
       </c>
       <c r="CN30" s="4">
-        <f>IF(COUNT(BY30:BY35)=6,ROUND((BY30/BY35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO30" s="4">
-        <f>IF(COUNT(CL30:CL49)=20,ROUND(STDEV(CL30:CL49),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP30" s="4">
+        <f>IF(COUNT(CF30:CF31)=2,ROUND((CF30/CF31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO30" s="5">
+        <f>IF(COUNT(CF30:CF31)=2,(CF30-CF31)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP30" s="3" t="n"/>
+      <c r="CQ30" s="4">
         <f>X30-P30</f>
         <v/>
       </c>
-      <c r="CQ30" s="4">
+      <c r="CR30" s="4">
         <f>AF30-P30</f>
         <v/>
       </c>
-      <c r="CR30" s="6">
-        <f>IF(COUNT(H30:H49)=20,CORREL(H30:H49,P30:P49),"")</f>
-        <v/>
-      </c>
-      <c r="CS30" s="4">
+      <c r="CS30" s="6">
+        <f>IF(COUNT(H30:H49)=20,IFERROR(CORREL(H30:H49,P30:P49),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT30" s="4">
         <f>AN30-AV30</f>
         <v/>
       </c>
-      <c r="CT30" s="4">
+      <c r="CU30" s="4">
         <f>BD30-BL30</f>
         <v/>
       </c>
-      <c r="CU30" s="6">
-        <f>BY30/CG30</f>
-        <v/>
-      </c>
-      <c r="CV30" s="4">
+      <c r="CV30" s="6">
+        <f>BY30/CF30</f>
+        <v/>
+      </c>
+      <c r="CW30" s="4">
         <f>P30-BT30</f>
         <v/>
       </c>
@@ -5851,75 +5860,76 @@
       <c r="CA31" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB31" s="4">
-        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC31" s="3" t="n"/>
+      <c r="CB31" s="3" t="n"/>
+      <c r="CC31" s="3" t="n">
+        <v>4.6</v>
+      </c>
       <c r="CD31" s="3" t="n">
-        <v>4.6</v>
+        <v>4.64</v>
       </c>
       <c r="CE31" s="3" t="n">
-        <v>4.64</v>
+        <v>4.598</v>
       </c>
       <c r="CF31" s="3" t="n">
-        <v>4.598</v>
+        <v>4.628</v>
       </c>
       <c r="CG31" s="3" t="n">
         <v>4.628</v>
       </c>
       <c r="CH31" s="3" t="n">
-        <v>4.628</v>
-      </c>
-      <c r="CI31" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI31" s="3" t="n"/>
       <c r="CJ31" s="4">
-        <f>IF(COUNT(CG31:CG32)=2,ROUND((CG31/CG32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK31" s="3" t="n"/>
+        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK31" s="4">
+        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL31" s="4">
-        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM31" s="5">
-        <f>IF(COUNT(CG31:CG32)=2,(CG31-CG32)*100,"")</f>
+        <f>IF(COUNT(BY31:BY36)=6,ROUND((BY31/BY36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM31" s="4">
+        <f>IF(COUNT(CK31:CK50)=20,IFERROR(ROUND(STDEV(CK31:CK50),4),""),"")</f>
         <v/>
       </c>
       <c r="CN31" s="4">
-        <f>IF(COUNT(BY31:BY36)=6,ROUND((BY31/BY36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO31" s="4">
-        <f>IF(COUNT(CL31:CL50)=20,ROUND(STDEV(CL31:CL50),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP31" s="4">
+        <f>IF(COUNT(CF31:CF32)=2,ROUND((CF31/CF32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO31" s="5">
+        <f>IF(COUNT(CF31:CF32)=2,(CF31-CF32)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP31" s="3" t="n"/>
+      <c r="CQ31" s="4">
         <f>X31-P31</f>
         <v/>
       </c>
-      <c r="CQ31" s="4">
+      <c r="CR31" s="4">
         <f>AF31-P31</f>
         <v/>
       </c>
-      <c r="CR31" s="6">
-        <f>IF(COUNT(H31:H50)=20,CORREL(H31:H50,P31:P50),"")</f>
-        <v/>
-      </c>
-      <c r="CS31" s="4">
+      <c r="CS31" s="6">
+        <f>IF(COUNT(H31:H50)=20,IFERROR(CORREL(H31:H50,P31:P50),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT31" s="4">
         <f>AN31-AV31</f>
         <v/>
       </c>
-      <c r="CT31" s="4">
+      <c r="CU31" s="4">
         <f>BD31-BL31</f>
         <v/>
       </c>
-      <c r="CU31" s="6">
-        <f>BY31/CG31</f>
-        <v/>
-      </c>
-      <c r="CV31" s="4">
+      <c r="CV31" s="6">
+        <f>BY31/CF31</f>
+        <v/>
+      </c>
+      <c r="CW31" s="4">
         <f>P31-BT31</f>
         <v/>
       </c>
@@ -6155,75 +6165,76 @@
       <c r="CA32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB32" s="4">
-        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC32" s="3" t="n"/>
+      <c r="CB32" s="3" t="n"/>
+      <c r="CC32" s="3" t="n">
+        <v>4.566</v>
+      </c>
       <c r="CD32" s="3" t="n">
-        <v>4.566</v>
+        <v>4.608</v>
       </c>
       <c r="CE32" s="3" t="n">
-        <v>4.608</v>
+        <v>4.56</v>
       </c>
       <c r="CF32" s="3" t="n">
-        <v>4.56</v>
+        <v>4.598</v>
       </c>
       <c r="CG32" s="3" t="n">
         <v>4.598</v>
       </c>
       <c r="CH32" s="3" t="n">
-        <v>4.598</v>
-      </c>
-      <c r="CI32" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI32" s="3" t="n"/>
       <c r="CJ32" s="4">
-        <f>IF(COUNT(CG32:CG33)=2,ROUND((CG32/CG33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK32" s="3" t="n"/>
+        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK32" s="4">
+        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL32" s="4">
-        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM32" s="5">
-        <f>IF(COUNT(CG32:CG33)=2,(CG32-CG33)*100,"")</f>
+        <f>IF(COUNT(BY32:BY37)=6,ROUND((BY32/BY37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM32" s="4">
+        <f>IF(COUNT(CK32:CK51)=20,IFERROR(ROUND(STDEV(CK32:CK51),4),""),"")</f>
         <v/>
       </c>
       <c r="CN32" s="4">
-        <f>IF(COUNT(BY32:BY37)=6,ROUND((BY32/BY37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO32" s="4">
-        <f>IF(COUNT(CL32:CL51)=20,ROUND(STDEV(CL32:CL51),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP32" s="4">
+        <f>IF(COUNT(CF32:CF33)=2,ROUND((CF32/CF33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO32" s="5">
+        <f>IF(COUNT(CF32:CF33)=2,(CF32-CF33)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP32" s="3" t="n"/>
+      <c r="CQ32" s="4">
         <f>X32-P32</f>
         <v/>
       </c>
-      <c r="CQ32" s="4">
+      <c r="CR32" s="4">
         <f>AF32-P32</f>
         <v/>
       </c>
-      <c r="CR32" s="6">
-        <f>IF(COUNT(H32:H51)=20,CORREL(H32:H51,P32:P51),"")</f>
-        <v/>
-      </c>
-      <c r="CS32" s="4">
+      <c r="CS32" s="6">
+        <f>IF(COUNT(H32:H51)=20,IFERROR(CORREL(H32:H51,P32:P51),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT32" s="4">
         <f>AN32-AV32</f>
         <v/>
       </c>
-      <c r="CT32" s="4">
+      <c r="CU32" s="4">
         <f>BD32-BL32</f>
         <v/>
       </c>
-      <c r="CU32" s="6">
-        <f>BY32/CG32</f>
-        <v/>
-      </c>
-      <c r="CV32" s="4">
+      <c r="CV32" s="6">
+        <f>BY32/CF32</f>
+        <v/>
+      </c>
+      <c r="CW32" s="4">
         <f>P32-BT32</f>
         <v/>
       </c>
@@ -6459,75 +6470,76 @@
       <c r="CA33" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB33" s="4">
-        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC33" s="3" t="n"/>
+      <c r="CB33" s="3" t="n"/>
+      <c r="CC33" s="3" t="n">
+        <v>4.521</v>
+      </c>
       <c r="CD33" s="3" t="n">
-        <v>4.521</v>
+        <v>4.55</v>
       </c>
       <c r="CE33" s="3" t="n">
-        <v>4.55</v>
+        <v>4.511</v>
       </c>
       <c r="CF33" s="3" t="n">
-        <v>4.511</v>
+        <v>4.541</v>
       </c>
       <c r="CG33" s="3" t="n">
         <v>4.541</v>
       </c>
       <c r="CH33" s="3" t="n">
-        <v>4.541</v>
-      </c>
-      <c r="CI33" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI33" s="3" t="n"/>
       <c r="CJ33" s="4">
-        <f>IF(COUNT(CG33:CG34)=2,ROUND((CG33/CG34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK33" s="3" t="n"/>
+        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK33" s="4">
+        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL33" s="4">
-        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM33" s="5">
-        <f>IF(COUNT(CG33:CG34)=2,(CG33-CG34)*100,"")</f>
+        <f>IF(COUNT(BY33:BY38)=6,ROUND((BY33/BY38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM33" s="4">
+        <f>IF(COUNT(CK33:CK52)=20,IFERROR(ROUND(STDEV(CK33:CK52),4),""),"")</f>
         <v/>
       </c>
       <c r="CN33" s="4">
-        <f>IF(COUNT(BY33:BY38)=6,ROUND((BY33/BY38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO33" s="4">
-        <f>IF(COUNT(CL33:CL52)=20,ROUND(STDEV(CL33:CL52),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP33" s="4">
+        <f>IF(COUNT(CF33:CF34)=2,ROUND((CF33/CF34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO33" s="5">
+        <f>IF(COUNT(CF33:CF34)=2,(CF33-CF34)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP33" s="3" t="n"/>
+      <c r="CQ33" s="4">
         <f>X33-P33</f>
         <v/>
       </c>
-      <c r="CQ33" s="4">
+      <c r="CR33" s="4">
         <f>AF33-P33</f>
         <v/>
       </c>
-      <c r="CR33" s="6">
-        <f>IF(COUNT(H33:H52)=20,CORREL(H33:H52,P33:P52),"")</f>
-        <v/>
-      </c>
-      <c r="CS33" s="4">
+      <c r="CS33" s="6">
+        <f>IF(COUNT(H33:H52)=20,IFERROR(CORREL(H33:H52,P33:P52),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT33" s="4">
         <f>AN33-AV33</f>
         <v/>
       </c>
-      <c r="CT33" s="4">
+      <c r="CU33" s="4">
         <f>BD33-BL33</f>
         <v/>
       </c>
-      <c r="CU33" s="6">
-        <f>BY33/CG33</f>
-        <v/>
-      </c>
-      <c r="CV33" s="4">
+      <c r="CV33" s="6">
+        <f>BY33/CF33</f>
+        <v/>
+      </c>
+      <c r="CW33" s="4">
         <f>P33-BT33</f>
         <v/>
       </c>
@@ -6763,75 +6775,76 @@
       <c r="CA34" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB34" s="4">
-        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC34" s="3" t="n"/>
+      <c r="CB34" s="3" t="n"/>
+      <c r="CC34" s="3" t="n">
+        <v>4.582</v>
+      </c>
       <c r="CD34" s="3" t="n">
-        <v>4.582</v>
+        <v>4.596</v>
       </c>
       <c r="CE34" s="3" t="n">
-        <v>4.596</v>
+        <v>4.561</v>
       </c>
       <c r="CF34" s="3" t="n">
-        <v>4.561</v>
+        <v>4.569</v>
       </c>
       <c r="CG34" s="3" t="n">
         <v>4.569</v>
       </c>
       <c r="CH34" s="3" t="n">
-        <v>4.569</v>
-      </c>
-      <c r="CI34" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI34" s="3" t="n"/>
       <c r="CJ34" s="4">
-        <f>IF(COUNT(CG34:CG35)=2,ROUND((CG34/CG35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK34" s="3" t="n"/>
+        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK34" s="4">
+        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL34" s="4">
-        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM34" s="5">
-        <f>IF(COUNT(CG34:CG35)=2,(CG34-CG35)*100,"")</f>
+        <f>IF(COUNT(BY34:BY39)=6,ROUND((BY34/BY39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM34" s="4">
+        <f>IF(COUNT(CK34:CK53)=20,IFERROR(ROUND(STDEV(CK34:CK53),4),""),"")</f>
         <v/>
       </c>
       <c r="CN34" s="4">
-        <f>IF(COUNT(BY34:BY39)=6,ROUND((BY34/BY39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO34" s="4">
-        <f>IF(COUNT(CL34:CL53)=20,ROUND(STDEV(CL34:CL53),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP34" s="4">
+        <f>IF(COUNT(CF34:CF35)=2,ROUND((CF34/CF35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO34" s="5">
+        <f>IF(COUNT(CF34:CF35)=2,(CF34-CF35)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP34" s="3" t="n"/>
+      <c r="CQ34" s="4">
         <f>X34-P34</f>
         <v/>
       </c>
-      <c r="CQ34" s="4">
+      <c r="CR34" s="4">
         <f>AF34-P34</f>
         <v/>
       </c>
-      <c r="CR34" s="6">
-        <f>IF(COUNT(H34:H53)=20,CORREL(H34:H53,P34:P53),"")</f>
-        <v/>
-      </c>
-      <c r="CS34" s="4">
+      <c r="CS34" s="6">
+        <f>IF(COUNT(H34:H53)=20,IFERROR(CORREL(H34:H53,P34:P53),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT34" s="4">
         <f>AN34-AV34</f>
         <v/>
       </c>
-      <c r="CT34" s="4">
+      <c r="CU34" s="4">
         <f>BD34-BL34</f>
         <v/>
       </c>
-      <c r="CU34" s="6">
-        <f>BY34/CG34</f>
-        <v/>
-      </c>
-      <c r="CV34" s="4">
+      <c r="CV34" s="6">
+        <f>BY34/CF34</f>
+        <v/>
+      </c>
+      <c r="CW34" s="4">
         <f>P34-BT34</f>
         <v/>
       </c>
@@ -7067,75 +7080,76 @@
       <c r="CA35" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB35" s="4">
-        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC35" s="3" t="n"/>
+      <c r="CB35" s="3" t="n"/>
+      <c r="CC35" s="3" t="n">
+        <v>4.608</v>
+      </c>
       <c r="CD35" s="3" t="n">
-        <v>4.608</v>
+        <v>4.61</v>
       </c>
       <c r="CE35" s="3" t="n">
-        <v>4.61</v>
+        <v>4.539</v>
       </c>
       <c r="CF35" s="3" t="n">
-        <v>4.539</v>
+        <v>4.545</v>
       </c>
       <c r="CG35" s="3" t="n">
         <v>4.545</v>
       </c>
       <c r="CH35" s="3" t="n">
-        <v>4.545</v>
-      </c>
-      <c r="CI35" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI35" s="3" t="n"/>
       <c r="CJ35" s="4">
-        <f>IF(COUNT(CG35:CG36)=2,ROUND((CG35/CG36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK35" s="3" t="n"/>
+        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK35" s="4">
+        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL35" s="4">
-        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM35" s="5">
-        <f>IF(COUNT(CG35:CG36)=2,(CG35-CG36)*100,"")</f>
+        <f>IF(COUNT(BY35:BY40)=6,ROUND((BY35/BY40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM35" s="4">
+        <f>IF(COUNT(CK35:CK54)=20,IFERROR(ROUND(STDEV(CK35:CK54),4),""),"")</f>
         <v/>
       </c>
       <c r="CN35" s="4">
-        <f>IF(COUNT(BY35:BY40)=6,ROUND((BY35/BY40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO35" s="4">
-        <f>IF(COUNT(CL35:CL54)=20,ROUND(STDEV(CL35:CL54),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP35" s="4">
+        <f>IF(COUNT(CF35:CF36)=2,ROUND((CF35/CF36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO35" s="5">
+        <f>IF(COUNT(CF35:CF36)=2,(CF35-CF36)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP35" s="3" t="n"/>
+      <c r="CQ35" s="4">
         <f>X35-P35</f>
         <v/>
       </c>
-      <c r="CQ35" s="4">
+      <c r="CR35" s="4">
         <f>AF35-P35</f>
         <v/>
       </c>
-      <c r="CR35" s="6">
-        <f>IF(COUNT(H35:H54)=20,CORREL(H35:H54,P35:P54),"")</f>
-        <v/>
-      </c>
-      <c r="CS35" s="4">
+      <c r="CS35" s="6">
+        <f>IF(COUNT(H35:H54)=20,IFERROR(CORREL(H35:H54,P35:P54),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT35" s="4">
         <f>AN35-AV35</f>
         <v/>
       </c>
-      <c r="CT35" s="4">
+      <c r="CU35" s="4">
         <f>BD35-BL35</f>
         <v/>
       </c>
-      <c r="CU35" s="6">
-        <f>BY35/CG35</f>
-        <v/>
-      </c>
-      <c r="CV35" s="4">
+      <c r="CV35" s="6">
+        <f>BY35/CF35</f>
+        <v/>
+      </c>
+      <c r="CW35" s="4">
         <f>P35-BT35</f>
         <v/>
       </c>
@@ -7371,75 +7385,76 @@
       <c r="CA36" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB36" s="4">
-        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC36" s="3" t="n"/>
+      <c r="CB36" s="3" t="n"/>
+      <c r="CC36" s="3" t="n">
+        <v>4.614</v>
+      </c>
       <c r="CD36" s="3" t="n">
         <v>4.614</v>
       </c>
       <c r="CE36" s="3" t="n">
-        <v>4.614</v>
+        <v>4.525</v>
       </c>
       <c r="CF36" s="3" t="n">
-        <v>4.525</v>
+        <v>4.585</v>
       </c>
       <c r="CG36" s="3" t="n">
         <v>4.585</v>
       </c>
       <c r="CH36" s="3" t="n">
-        <v>4.585</v>
-      </c>
-      <c r="CI36" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI36" s="3" t="n"/>
       <c r="CJ36" s="4">
-        <f>IF(COUNT(CG36:CG37)=2,ROUND((CG36/CG37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK36" s="3" t="n"/>
+        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK36" s="4">
+        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL36" s="4">
-        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM36" s="5">
-        <f>IF(COUNT(CG36:CG37)=2,(CG36-CG37)*100,"")</f>
+        <f>IF(COUNT(BY36:BY41)=6,ROUND((BY36/BY41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM36" s="4">
+        <f>IF(COUNT(CK36:CK55)=20,IFERROR(ROUND(STDEV(CK36:CK55),4),""),"")</f>
         <v/>
       </c>
       <c r="CN36" s="4">
-        <f>IF(COUNT(BY36:BY41)=6,ROUND((BY36/BY41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO36" s="4">
-        <f>IF(COUNT(CL36:CL55)=20,ROUND(STDEV(CL36:CL55),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP36" s="4">
+        <f>IF(COUNT(CF36:CF37)=2,ROUND((CF36/CF37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO36" s="5">
+        <f>IF(COUNT(CF36:CF37)=2,(CF36-CF37)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP36" s="3" t="n"/>
+      <c r="CQ36" s="4">
         <f>X36-P36</f>
         <v/>
       </c>
-      <c r="CQ36" s="4">
+      <c r="CR36" s="4">
         <f>AF36-P36</f>
         <v/>
       </c>
-      <c r="CR36" s="6">
-        <f>IF(COUNT(H36:H55)=20,CORREL(H36:H55,P36:P55),"")</f>
-        <v/>
-      </c>
-      <c r="CS36" s="4">
+      <c r="CS36" s="6">
+        <f>IF(COUNT(H36:H55)=20,IFERROR(CORREL(H36:H55,P36:P55),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT36" s="4">
         <f>AN36-AV36</f>
         <v/>
       </c>
-      <c r="CT36" s="4">
+      <c r="CU36" s="4">
         <f>BD36-BL36</f>
         <v/>
       </c>
-      <c r="CU36" s="6">
-        <f>BY36/CG36</f>
-        <v/>
-      </c>
-      <c r="CV36" s="4">
+      <c r="CV36" s="6">
+        <f>BY36/CF36</f>
+        <v/>
+      </c>
+      <c r="CW36" s="4">
         <f>P36-BT36</f>
         <v/>
       </c>
@@ -7675,75 +7690,76 @@
       <c r="CA37" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB37" s="4">
-        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC37" s="3" t="n"/>
+      <c r="CB37" s="3" t="n"/>
+      <c r="CC37" s="3" t="n">
+        <v>4.585</v>
+      </c>
       <c r="CD37" s="3" t="n">
-        <v>4.585</v>
+        <v>4.618</v>
       </c>
       <c r="CE37" s="3" t="n">
-        <v>4.618</v>
+        <v>4.573</v>
       </c>
       <c r="CF37" s="3" t="n">
-        <v>4.573</v>
+        <v>4.609</v>
       </c>
       <c r="CG37" s="3" t="n">
         <v>4.609</v>
       </c>
       <c r="CH37" s="3" t="n">
-        <v>4.609</v>
-      </c>
-      <c r="CI37" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI37" s="3" t="n"/>
       <c r="CJ37" s="4">
-        <f>IF(COUNT(CG37:CG38)=2,ROUND((CG37/CG38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK37" s="3" t="n"/>
+        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK37" s="4">
+        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
+        <v/>
+      </c>
       <c r="CL37" s="4">
-        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CM37" s="5">
-        <f>IF(COUNT(CG37:CG38)=2,(CG37-CG38)*100,"")</f>
+        <f>IF(COUNT(BY37:BY42)=6,ROUND((BY37/BY42-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CM37" s="4">
+        <f>IF(COUNT(CK37:CK56)=20,IFERROR(ROUND(STDEV(CK37:CK56),4),""),"")</f>
         <v/>
       </c>
       <c r="CN37" s="4">
-        <f>IF(COUNT(BY37:BY42)=6,ROUND((BY37/BY42-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO37" s="4">
-        <f>IF(COUNT(CL37:CL56)=20,ROUND(STDEV(CL37:CL56),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP37" s="4">
+        <f>IF(COUNT(CF37:CF38)=2,ROUND((CF37/CF38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO37" s="5">
+        <f>IF(COUNT(CF37:CF38)=2,(CF37-CF38)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP37" s="3" t="n"/>
+      <c r="CQ37" s="4">
         <f>X37-P37</f>
         <v/>
       </c>
-      <c r="CQ37" s="4">
+      <c r="CR37" s="4">
         <f>AF37-P37</f>
         <v/>
       </c>
-      <c r="CR37" s="6">
-        <f>IF(COUNT(H37:H56)=20,CORREL(H37:H56,P37:P56),"")</f>
-        <v/>
-      </c>
-      <c r="CS37" s="4">
+      <c r="CS37" s="6">
+        <f>IF(COUNT(H37:H56)=20,IFERROR(CORREL(H37:H56,P37:P56),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT37" s="4">
         <f>AN37-AV37</f>
         <v/>
       </c>
-      <c r="CT37" s="4">
+      <c r="CU37" s="4">
         <f>BD37-BL37</f>
         <v/>
       </c>
-      <c r="CU37" s="6">
-        <f>BY37/CG37</f>
-        <v/>
-      </c>
-      <c r="CV37" s="4">
+      <c r="CV37" s="6">
+        <f>BY37/CF37</f>
+        <v/>
+      </c>
+      <c r="CW37" s="4">
         <f>P37-BT37</f>
         <v/>
       </c>
@@ -7979,72 +7995,73 @@
       <c r="CA38" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB38" s="4">
-        <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC38" s="3" t="n"/>
+      <c r="CB38" s="3" t="n"/>
+      <c r="CC38" s="3" t="n">
+        <v>4.541</v>
+      </c>
       <c r="CD38" s="3" t="n">
-        <v>4.541</v>
+        <v>4.571</v>
       </c>
       <c r="CE38" s="3" t="n">
-        <v>4.571</v>
+        <v>4.539</v>
       </c>
       <c r="CF38" s="3" t="n">
-        <v>4.539</v>
+        <v>4.569</v>
       </c>
       <c r="CG38" s="3" t="n">
         <v>4.569</v>
       </c>
       <c r="CH38" s="3" t="n">
-        <v>4.569</v>
-      </c>
-      <c r="CI38" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI38" s="3" t="n"/>
       <c r="CJ38" s="4">
-        <f>IF(COUNT(CG38:CG39)=2,ROUND((CG38/CG39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK38" s="3" t="n"/>
-      <c r="CL38" s="4">
         <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="CM38" s="5">
-        <f>IF(COUNT(CG38:CG39)=2,(CG38-CG39)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CN38" s="4" t="n"/>
-      <c r="CO38" s="4">
-        <f>IF(COUNT(CL38:CL57)=20,ROUND(STDEV(CL38:CL57),4),"")</f>
-        <v/>
-      </c>
-      <c r="CP38" s="4">
+      <c r="CK38" s="4">
+        <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CL38" s="4" t="n"/>
+      <c r="CM38" s="4">
+        <f>IF(COUNT(CK38:CK57)=20,IFERROR(ROUND(STDEV(CK38:CK57),4),""),"")</f>
+        <v/>
+      </c>
+      <c r="CN38" s="4">
+        <f>IF(COUNT(CF38:CF39)=2,ROUND((CF38/CF39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO38" s="5">
+        <f>IF(COUNT(CF38:CF39)=2,(CF38-CF39)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP38" s="3" t="n"/>
+      <c r="CQ38" s="4">
         <f>X38-P38</f>
         <v/>
       </c>
-      <c r="CQ38" s="4">
+      <c r="CR38" s="4">
         <f>AF38-P38</f>
         <v/>
       </c>
-      <c r="CR38" s="6">
-        <f>IF(COUNT(H38:H57)=20,CORREL(H38:H57,P38:P57),"")</f>
-        <v/>
-      </c>
-      <c r="CS38" s="4">
+      <c r="CS38" s="6">
+        <f>IF(COUNT(H38:H57)=20,IFERROR(CORREL(H38:H57,P38:P57),""),"")</f>
+        <v/>
+      </c>
+      <c r="CT38" s="4">
         <f>AN38-AV38</f>
         <v/>
       </c>
-      <c r="CT38" s="4">
+      <c r="CU38" s="4">
         <f>BD38-BL38</f>
         <v/>
       </c>
-      <c r="CU38" s="6">
-        <f>BY38/CG38</f>
-        <v/>
-      </c>
-      <c r="CV38" s="4">
+      <c r="CV38" s="6">
+        <f>BY38/CF38</f>
+        <v/>
+      </c>
+      <c r="CW38" s="4">
         <f>P38-BT38</f>
         <v/>
       </c>
@@ -8280,66 +8297,67 @@
       <c r="CA39" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB39" s="4">
-        <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC39" s="3" t="n"/>
+      <c r="CB39" s="3" t="n"/>
+      <c r="CC39" s="3" t="n">
+        <v>4.577</v>
+      </c>
       <c r="CD39" s="3" t="n">
-        <v>4.577</v>
+        <v>4.581</v>
       </c>
       <c r="CE39" s="3" t="n">
-        <v>4.581</v>
+        <v>4.529</v>
       </c>
       <c r="CF39" s="3" t="n">
-        <v>4.529</v>
+        <v>4.539</v>
       </c>
       <c r="CG39" s="3" t="n">
         <v>4.539</v>
       </c>
       <c r="CH39" s="3" t="n">
-        <v>4.539</v>
-      </c>
-      <c r="CI39" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI39" s="3" t="n"/>
       <c r="CJ39" s="4">
-        <f>IF(COUNT(CG39:CG40)=2,ROUND((CG39/CG40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK39" s="3" t="n"/>
-      <c r="CL39" s="4">
         <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="CM39" s="5">
-        <f>IF(COUNT(CG39:CG40)=2,(CG39-CG40)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CN39" s="4" t="n"/>
-      <c r="CO39" s="4" t="n"/>
-      <c r="CP39" s="4">
+      <c r="CK39" s="4">
+        <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CL39" s="4" t="n"/>
+      <c r="CM39" s="4" t="n"/>
+      <c r="CN39" s="4">
+        <f>IF(COUNT(CF39:CF40)=2,ROUND((CF39/CF40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO39" s="5">
+        <f>IF(COUNT(CF39:CF40)=2,(CF39-CF40)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP39" s="3" t="n"/>
+      <c r="CQ39" s="4">
         <f>X39-P39</f>
         <v/>
       </c>
-      <c r="CQ39" s="4">
+      <c r="CR39" s="4">
         <f>AF39-P39</f>
         <v/>
       </c>
-      <c r="CR39" s="6" t="n"/>
-      <c r="CS39" s="4">
+      <c r="CS39" s="6" t="n"/>
+      <c r="CT39" s="4">
         <f>AN39-AV39</f>
         <v/>
       </c>
-      <c r="CT39" s="4">
+      <c r="CU39" s="4">
         <f>BD39-BL39</f>
         <v/>
       </c>
-      <c r="CU39" s="6">
-        <f>BY39/CG39</f>
-        <v/>
-      </c>
-      <c r="CV39" s="4">
+      <c r="CV39" s="6">
+        <f>BY39/CF39</f>
+        <v/>
+      </c>
+      <c r="CW39" s="4">
         <f>P39-BT39</f>
         <v/>
       </c>
@@ -8575,66 +8593,67 @@
       <c r="CA40" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB40" s="4">
-        <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC40" s="3" t="n"/>
+      <c r="CB40" s="3" t="n"/>
+      <c r="CC40" s="3" t="n">
+        <v>4.561</v>
+      </c>
       <c r="CD40" s="3" t="n">
-        <v>4.561</v>
+        <v>4.597</v>
       </c>
       <c r="CE40" s="3" t="n">
-        <v>4.597</v>
+        <v>4.557</v>
       </c>
       <c r="CF40" s="3" t="n">
-        <v>4.557</v>
+        <v>4.569</v>
       </c>
       <c r="CG40" s="3" t="n">
         <v>4.569</v>
       </c>
       <c r="CH40" s="3" t="n">
-        <v>4.569</v>
-      </c>
-      <c r="CI40" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI40" s="3" t="n"/>
       <c r="CJ40" s="4">
-        <f>IF(COUNT(CG40:CG41)=2,ROUND((CG40/CG41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK40" s="3" t="n"/>
-      <c r="CL40" s="4">
         <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="CM40" s="5">
-        <f>IF(COUNT(CG40:CG41)=2,(CG40-CG41)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CN40" s="4" t="n"/>
-      <c r="CO40" s="4" t="n"/>
-      <c r="CP40" s="4">
+      <c r="CK40" s="4">
+        <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CL40" s="4" t="n"/>
+      <c r="CM40" s="4" t="n"/>
+      <c r="CN40" s="4">
+        <f>IF(COUNT(CF40:CF41)=2,ROUND((CF40/CF41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO40" s="5">
+        <f>IF(COUNT(CF40:CF41)=2,(CF40-CF41)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP40" s="3" t="n"/>
+      <c r="CQ40" s="4">
         <f>X40-P40</f>
         <v/>
       </c>
-      <c r="CQ40" s="4">
+      <c r="CR40" s="4">
         <f>AF40-P40</f>
         <v/>
       </c>
-      <c r="CR40" s="6" t="n"/>
-      <c r="CS40" s="4">
+      <c r="CS40" s="6" t="n"/>
+      <c r="CT40" s="4">
         <f>AN40-AV40</f>
         <v/>
       </c>
-      <c r="CT40" s="4">
+      <c r="CU40" s="4">
         <f>BD40-BL40</f>
         <v/>
       </c>
-      <c r="CU40" s="6">
-        <f>BY40/CG40</f>
-        <v/>
-      </c>
-      <c r="CV40" s="4">
+      <c r="CV40" s="6">
+        <f>BY40/CF40</f>
+        <v/>
+      </c>
+      <c r="CW40" s="4">
         <f>P40-BT40</f>
         <v/>
       </c>
@@ -8870,66 +8889,67 @@
       <c r="CA41" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB41" s="4">
-        <f>IF(COUNT(BY41:BY42)=2,ROUND((BY41/BY42-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CC41" s="3" t="n"/>
+      <c r="CB41" s="3" t="n"/>
+      <c r="CC41" s="3" t="n">
+        <v>4.497</v>
+      </c>
       <c r="CD41" s="3" t="n">
-        <v>4.497</v>
+        <v>4.533</v>
       </c>
       <c r="CE41" s="3" t="n">
-        <v>4.533</v>
+        <v>4.485</v>
       </c>
       <c r="CF41" s="3" t="n">
-        <v>4.485</v>
+        <v>4.529</v>
       </c>
       <c r="CG41" s="3" t="n">
         <v>4.529</v>
       </c>
       <c r="CH41" s="3" t="n">
-        <v>4.529</v>
-      </c>
-      <c r="CI41" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="CI41" s="3" t="n"/>
       <c r="CJ41" s="4">
-        <f>IF(COUNT(CG41:CG42)=2,ROUND((CG41/CG42-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK41" s="3" t="n"/>
-      <c r="CL41" s="4">
         <f>IF(COUNT(BY41:BY42)=2,ROUND((BY41/BY42-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="CM41" s="5">
-        <f>IF(COUNT(CG41:CG42)=2,(CG41-CG42)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CN41" s="4" t="n"/>
-      <c r="CO41" s="4" t="n"/>
-      <c r="CP41" s="4">
+      <c r="CK41" s="4">
+        <f>IF(COUNT(BY41:BY42)=2,ROUND((BY41/BY42-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CL41" s="4" t="n"/>
+      <c r="CM41" s="4" t="n"/>
+      <c r="CN41" s="4">
+        <f>IF(COUNT(CF41:CF42)=2,ROUND((CF41/CF42-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO41" s="5">
+        <f>IF(COUNT(CF41:CF42)=2,(CF41-CF42)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP41" s="3" t="n"/>
+      <c r="CQ41" s="4">
         <f>X41-P41</f>
         <v/>
       </c>
-      <c r="CQ41" s="4">
+      <c r="CR41" s="4">
         <f>AF41-P41</f>
         <v/>
       </c>
-      <c r="CR41" s="6" t="n"/>
-      <c r="CS41" s="4">
+      <c r="CS41" s="6" t="n"/>
+      <c r="CT41" s="4">
         <f>AN41-AV41</f>
         <v/>
       </c>
-      <c r="CT41" s="4">
+      <c r="CU41" s="4">
         <f>BD41-BL41</f>
         <v/>
       </c>
-      <c r="CU41" s="6">
-        <f>BY41/CG41</f>
-        <v/>
-      </c>
-      <c r="CV41" s="4">
+      <c r="CV41" s="6">
+        <f>BY41/CF41</f>
+        <v/>
+      </c>
+      <c r="CW41" s="4">
         <f>P41-BT41</f>
         <v/>
       </c>
@@ -9138,60 +9158,67 @@
       <c r="CA42" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CB42" s="4" t="n"/>
-      <c r="CC42" s="3" t="n"/>
+      <c r="CB42" s="3" t="n"/>
+      <c r="CC42" s="3" t="n">
+        <v>4.457</v>
+      </c>
       <c r="CD42" s="3" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="CE42" s="3" t="n">
         <v>4.457</v>
       </c>
-      <c r="CE42" s="3" t="n">
-        <v>4.491</v>
-      </c>
       <c r="CF42" s="3" t="n">
-        <v>4.457</v>
+        <v>4.479</v>
       </c>
       <c r="CG42" s="3" t="n">
         <v>4.479</v>
       </c>
       <c r="CH42" s="3" t="n">
-        <v>4.479</v>
-      </c>
-      <c r="CI42" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="CJ42" s="4" t="n"/>
-      <c r="CK42" s="3" t="n"/>
-      <c r="CL42" s="4">
+      <c r="CI42" s="3" t="n"/>
+      <c r="CJ42" s="4">
         <f>IF(COUNT(BY42:BY43)=2,ROUND((BY42/BY43-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="CM42" s="5">
-        <f>IF(COUNT(CG42:CG43)=2,(CG42-CG43)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CN42" s="4" t="n"/>
-      <c r="CO42" s="4" t="n"/>
-      <c r="CP42" s="4">
+      <c r="CK42" s="4">
+        <f>IF(COUNT(BY42:BY43)=2,ROUND((BY42/BY43-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CL42" s="4" t="n"/>
+      <c r="CM42" s="4" t="n"/>
+      <c r="CN42" s="4">
+        <f>IF(COUNT(CF42:CF43)=2,ROUND((CF42/CF43-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CO42" s="5">
+        <f>IF(COUNT(CF42:CF43)=2,(CF42-CF43)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CP42" s="3" t="n"/>
+      <c r="CQ42" s="4">
         <f>X42-P42</f>
         <v/>
       </c>
-      <c r="CQ42" s="4">
+      <c r="CR42" s="4">
         <f>AF42-P42</f>
         <v/>
       </c>
-      <c r="CR42" s="6" t="n"/>
-      <c r="CS42" s="4">
+      <c r="CS42" s="6" t="n"/>
+      <c r="CT42" s="4">
         <f>AN42-AV42</f>
         <v/>
       </c>
-      <c r="CT42" s="4">
+      <c r="CU42" s="4">
         <f>BD42-BL42</f>
         <v/>
       </c>
-      <c r="CU42" s="6">
-        <f>BY42/CG42</f>
-        <v/>
-      </c>
-      <c r="CV42" s="4">
+      <c r="CV42" s="6">
+        <f>BY42/CF42</f>
+        <v/>
+      </c>
+      <c r="CW42" s="4">
         <f>P42-BT42</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
data: fetch VIX/TNX OHLC and refresh external sample
</commit_message>
<xml_diff>
--- a/04_结果/示例审批/外部数据新版式示例.xlsx
+++ b/04_结果/示例审批/外部数据新版式示例.xlsx
@@ -490,7 +490,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1. VIX/TNX 原始数据按 ETF 格式展示：第14行=名称，第15行=Open/High/Low/Close/Adj Close/Volume。</t>
+          <t>1. VIX/TNX 原始数据按 ETF 格式展示：第14行=名称，第15行=Open/High/Low/Close（只保留 OHLC，不展示 Adj Close/Volume）。</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A14:CW40"/>
+  <dimension ref="A14:CS40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -626,10 +626,6 @@
     <col width="14" customWidth="1" min="95" max="95"/>
     <col width="14" customWidth="1" min="96" max="96"/>
     <col width="14" customWidth="1" min="97" max="97"/>
-    <col width="14" customWidth="1" min="98" max="98"/>
-    <col width="14" customWidth="1" min="99" max="99"/>
-    <col width="14" customWidth="1" min="100" max="100"/>
-    <col width="14" customWidth="1" min="101" max="101"/>
   </cols>
   <sheetData>
     <row r="14" ht="30" customHeight="1">
@@ -757,71 +753,67 @@
       <c r="BZ14" s="2" t="n"/>
       <c r="CA14" s="2" t="n"/>
       <c r="CB14" s="2" t="n"/>
-      <c r="CC14" s="2" t="n"/>
+      <c r="CC14" s="2" t="inlineStr">
+        <is>
+          <t>TNX</t>
+        </is>
+      </c>
       <c r="CD14" s="2" t="n"/>
-      <c r="CE14" s="2" t="inlineStr">
-        <is>
-          <t>TNX</t>
-        </is>
-      </c>
+      <c r="CE14" s="2" t="n"/>
       <c r="CF14" s="2" t="n"/>
-      <c r="CG14" s="2" t="n"/>
-      <c r="CH14" s="2" t="n"/>
-      <c r="CI14" s="2" t="n"/>
+      <c r="CG14" s="2" t="inlineStr">
+        <is>
+          <t>VIX_Chg%</t>
+        </is>
+      </c>
+      <c r="CH14" s="2" t="inlineStr">
+        <is>
+          <t>VIX_5dChg</t>
+        </is>
+      </c>
+      <c r="CI14" s="2" t="inlineStr">
+        <is>
+          <t>VIX_20dVol</t>
+        </is>
+      </c>
       <c r="CJ14" s="2" t="n"/>
       <c r="CK14" s="2" t="inlineStr">
         <is>
-          <t>VIX_Chg%</t>
-        </is>
-      </c>
-      <c r="CL14" s="2" t="inlineStr">
-        <is>
-          <t>VIX_5dChg</t>
-        </is>
-      </c>
+          <t>TNX_ChgBp</t>
+        </is>
+      </c>
+      <c r="CL14" s="2" t="n"/>
       <c r="CM14" s="2" t="inlineStr">
         <is>
-          <t>VIX_20dVol</t>
-        </is>
-      </c>
-      <c r="CN14" s="2" t="n"/>
+          <t>CreditSpread</t>
+        </is>
+      </c>
+      <c r="CN14" s="2" t="inlineStr">
+        <is>
+          <t>JNKSpread</t>
+        </is>
+      </c>
       <c r="CO14" s="2" t="inlineStr">
         <is>
-          <t>TNX_ChgBp</t>
-        </is>
-      </c>
-      <c r="CP14" s="2" t="n"/>
+          <t>StkBonCorr</t>
+        </is>
+      </c>
+      <c r="CP14" s="2" t="inlineStr">
+        <is>
+          <t>USDGoldRatio</t>
+        </is>
+      </c>
       <c r="CQ14" s="2" t="inlineStr">
         <is>
-          <t>CreditSpread</t>
+          <t>SectRotation</t>
         </is>
       </c>
       <c r="CR14" s="2" t="inlineStr">
         <is>
-          <t>JNKSpread</t>
+          <t>VIX_TNX_Ratio</t>
         </is>
       </c>
       <c r="CS14" s="2" t="inlineStr">
-        <is>
-          <t>StkBonCorr</t>
-        </is>
-      </c>
-      <c r="CT14" s="2" t="inlineStr">
-        <is>
-          <t>USDGoldRatio</t>
-        </is>
-      </c>
-      <c r="CU14" s="2" t="inlineStr">
-        <is>
-          <t>SectRotation</t>
-        </is>
-      </c>
-      <c r="CV14" s="2" t="inlineStr">
-        <is>
-          <t>VIX_TNX_Ratio</t>
-        </is>
-      </c>
-      <c r="CW14" s="2" t="inlineStr">
         <is>
           <t>YldCurveProxy</t>
         </is>
@@ -1177,110 +1169,90 @@
           <t>Close</t>
         </is>
       </c>
-      <c r="BZ15" s="2" t="inlineStr">
-        <is>
-          <t>Adj Close</t>
-        </is>
-      </c>
+      <c r="BZ15" s="2" t="n"/>
       <c r="CA15" s="2" t="inlineStr">
         <is>
-          <t>Volume</t>
-        </is>
-      </c>
-      <c r="CB15" s="2" t="n"/>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="CB15" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="CC15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="CD15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="CE15" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="CE15" s="2" t="n"/>
       <c r="CF15" s="2" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>VIX回报</t>
         </is>
       </c>
       <c r="CG15" s="2" t="inlineStr">
         <is>
-          <t>Adj Close</t>
+          <t>VIX_close/昨VIX_close-1</t>
         </is>
       </c>
       <c r="CH15" s="2" t="inlineStr">
         <is>
-          <t>Volume</t>
-        </is>
-      </c>
-      <c r="CI15" s="2" t="n"/>
+          <t>VIX_close/5日前VIX_close-1</t>
+        </is>
+      </c>
+      <c r="CI15" s="2" t="inlineStr">
+        <is>
+          <t>STDEV(VIX日变化,近20日)</t>
+        </is>
+      </c>
       <c r="CJ15" s="2" t="inlineStr">
         <is>
-          <t>VIX回报</t>
+          <t>TNX回报</t>
         </is>
       </c>
       <c r="CK15" s="2" t="inlineStr">
         <is>
-          <t>VIX_close/昨VIX_close-1</t>
-        </is>
-      </c>
-      <c r="CL15" s="2" t="inlineStr">
-        <is>
-          <t>VIX_close/5日前VIX_close-1</t>
-        </is>
-      </c>
+          <t>(TNX_close-昨TNX_close)*100</t>
+        </is>
+      </c>
+      <c r="CL15" s="2" t="n"/>
       <c r="CM15" s="2" t="inlineStr">
         <is>
-          <t>STDEV(VIX日变化,近20日)</t>
+          <t>HYG-TLT</t>
         </is>
       </c>
       <c r="CN15" s="2" t="inlineStr">
         <is>
-          <t>TNX回报</t>
+          <t>JNK-TLT</t>
         </is>
       </c>
       <c r="CO15" s="2" t="inlineStr">
         <is>
-          <t>(TNX_close-昨TNX_close)*100</t>
-        </is>
-      </c>
-      <c r="CP15" s="2" t="n"/>
+          <t>CORREL(SPY,TLT,近20日)</t>
+        </is>
+      </c>
+      <c r="CP15" s="2" t="inlineStr">
+        <is>
+          <t>UUP-GLD</t>
+        </is>
+      </c>
       <c r="CQ15" s="2" t="inlineStr">
         <is>
-          <t>HYG-TLT</t>
+          <t>XLK-XLF</t>
         </is>
       </c>
       <c r="CR15" s="2" t="inlineStr">
         <is>
-          <t>JNK-TLT</t>
+          <t>VIX_close/TNX_close</t>
         </is>
       </c>
       <c r="CS15" s="2" t="inlineStr">
-        <is>
-          <t>CORREL(SPY,TLT,近20日)</t>
-        </is>
-      </c>
-      <c r="CT15" s="2" t="inlineStr">
-        <is>
-          <t>UUP-GLD</t>
-        </is>
-      </c>
-      <c r="CU15" s="2" t="inlineStr">
-        <is>
-          <t>XLK-XLF</t>
-        </is>
-      </c>
-      <c r="CV15" s="2" t="inlineStr">
-        <is>
-          <t>VIX_close/TNX_close</t>
-        </is>
-      </c>
-      <c r="CW15" s="2" t="inlineStr">
         <is>
           <t>TLT-TIP</t>
         </is>
@@ -1511,82 +1483,70 @@
       <c r="BY16" s="3" t="n">
         <v>14.9</v>
       </c>
-      <c r="BZ16" s="3" t="n">
-        <v>14.9</v>
-      </c>
+      <c r="BZ16" s="3" t="n"/>
       <c r="CA16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB16" s="3" t="n"/>
+        <v>4.664</v>
+      </c>
+      <c r="CB16" s="3" t="n">
+        <v>4.672</v>
+      </c>
       <c r="CC16" s="3" t="n">
-        <v>4.664</v>
+        <v>4.603</v>
       </c>
       <c r="CD16" s="3" t="n">
-        <v>4.672</v>
-      </c>
-      <c r="CE16" s="3" t="n">
-        <v>4.603</v>
-      </c>
-      <c r="CF16" s="3" t="n">
         <v>4.66</v>
       </c>
-      <c r="CG16" s="3" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="CH16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI16" s="3" t="n"/>
+      <c r="CE16" s="3" t="n"/>
+      <c r="CF16" s="4">
+        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG16" s="4">
+        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH16" s="4">
+        <f>IF(COUNT(BY16:BY21)=6,ROUND((BY16/BY21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI16" s="4">
+        <f>IF(COUNT(CG16:CG35)=20,IFERROR(ROUND(STDEV(CG16:CG35),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ16" s="4">
-        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK16" s="4">
-        <f>IF(COUNT(BY16:BY17)=2,ROUND((BY16/BY17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL16" s="4">
-        <f>IF(COUNT(BY16:BY21)=6,ROUND((BY16/BY21-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD16:CD17)=2,ROUND((CD16/CD17-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK16" s="5">
+        <f>IF(COUNT(CD16:CD17)=2,(CD16-CD17)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL16" s="3" t="n"/>
       <c r="CM16" s="4">
-        <f>IF(COUNT(CK16:CK35)=20,IFERROR(ROUND(STDEV(CK16:CK35),4),""),"")</f>
+        <f>IFERROR(X16-P16,"")</f>
         <v/>
       </c>
       <c r="CN16" s="4">
-        <f>IF(COUNT(CF16:CF17)=2,ROUND((CF16/CF17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO16" s="5">
-        <f>IF(COUNT(CF16:CF17)=2,(CF16-CF17)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP16" s="3" t="n"/>
+        <f>IFERROR(AF16-P16,"")</f>
+        <v/>
+      </c>
+      <c r="CO16" s="6">
+        <f>IF(COUNT(H16:H35)=20,IFERROR(CORREL(H16:H35,P16:P35),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP16" s="4">
+        <f>IFERROR(AN16-AV16,"")</f>
+        <v/>
+      </c>
       <c r="CQ16" s="4">
-        <f>IFERROR(X16-P16,"")</f>
-        <v/>
-      </c>
-      <c r="CR16" s="4">
-        <f>IFERROR(AF16-P16,"")</f>
-        <v/>
-      </c>
-      <c r="CS16" s="6">
-        <f>IF(COUNT(H16:H35)=20,IFERROR(CORREL(H16:H35,P16:P35),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT16" s="4">
-        <f>IFERROR(AN16-AV16,"")</f>
-        <v/>
-      </c>
-      <c r="CU16" s="4">
         <f>IFERROR(BD16-BL16,"")</f>
         <v/>
       </c>
-      <c r="CV16" s="6">
-        <f>BY16/CF16</f>
-        <v/>
-      </c>
-      <c r="CW16" s="4">
+      <c r="CR16" s="6">
+        <f>BY16/CD16</f>
+        <v/>
+      </c>
+      <c r="CS16" s="4">
         <f>IFERROR(P16-BT16,"")</f>
         <v/>
       </c>
@@ -1816,82 +1776,70 @@
       <c r="BY17" s="3" t="n">
         <v>15.15</v>
       </c>
-      <c r="BZ17" s="3" t="n">
-        <v>15.15</v>
-      </c>
+      <c r="BZ17" s="3" t="n"/>
       <c r="CA17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB17" s="3" t="n"/>
+        <v>4.643</v>
+      </c>
+      <c r="CB17" s="3" t="n">
+        <v>4.676</v>
+      </c>
       <c r="CC17" s="3" t="n">
-        <v>4.643</v>
+        <v>4.635</v>
       </c>
       <c r="CD17" s="3" t="n">
-        <v>4.676</v>
-      </c>
-      <c r="CE17" s="3" t="n">
-        <v>4.635</v>
-      </c>
-      <c r="CF17" s="3" t="n">
         <v>4.67</v>
       </c>
-      <c r="CG17" s="3" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="CH17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI17" s="3" t="n"/>
+      <c r="CE17" s="3" t="n"/>
+      <c r="CF17" s="4">
+        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG17" s="4">
+        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH17" s="4">
+        <f>IF(COUNT(BY17:BY22)=6,ROUND((BY17/BY22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI17" s="4">
+        <f>IF(COUNT(CG17:CG36)=20,IFERROR(ROUND(STDEV(CG17:CG36),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ17" s="4">
-        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK17" s="4">
-        <f>IF(COUNT(BY17:BY18)=2,ROUND((BY17/BY18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL17" s="4">
-        <f>IF(COUNT(BY17:BY22)=6,ROUND((BY17/BY22-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD17:CD18)=2,ROUND((CD17/CD18-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK17" s="5">
+        <f>IF(COUNT(CD17:CD18)=2,(CD17-CD18)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL17" s="3" t="n"/>
       <c r="CM17" s="4">
-        <f>IF(COUNT(CK17:CK36)=20,IFERROR(ROUND(STDEV(CK17:CK36),4),""),"")</f>
+        <f>IFERROR(X17-P17,"")</f>
         <v/>
       </c>
       <c r="CN17" s="4">
-        <f>IF(COUNT(CF17:CF18)=2,ROUND((CF17/CF18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO17" s="5">
-        <f>IF(COUNT(CF17:CF18)=2,(CF17-CF18)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP17" s="3" t="n"/>
+        <f>IFERROR(AF17-P17,"")</f>
+        <v/>
+      </c>
+      <c r="CO17" s="6">
+        <f>IF(COUNT(H17:H36)=20,IFERROR(CORREL(H17:H36,P17:P36),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP17" s="4">
+        <f>IFERROR(AN17-AV17,"")</f>
+        <v/>
+      </c>
       <c r="CQ17" s="4">
-        <f>IFERROR(X17-P17,"")</f>
-        <v/>
-      </c>
-      <c r="CR17" s="4">
-        <f>IFERROR(AF17-P17,"")</f>
-        <v/>
-      </c>
-      <c r="CS17" s="6">
-        <f>IF(COUNT(H17:H36)=20,IFERROR(CORREL(H17:H36,P17:P36),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT17" s="4">
-        <f>IFERROR(AN17-AV17,"")</f>
-        <v/>
-      </c>
-      <c r="CU17" s="4">
         <f>IFERROR(BD17-BL17,"")</f>
         <v/>
       </c>
-      <c r="CV17" s="6">
-        <f>BY17/CF17</f>
-        <v/>
-      </c>
-      <c r="CW17" s="4">
+      <c r="CR17" s="6">
+        <f>BY17/CD17</f>
+        <v/>
+      </c>
+      <c r="CS17" s="4">
         <f>IFERROR(P17-BT17,"")</f>
         <v/>
       </c>
@@ -2121,82 +2069,70 @@
       <c r="BY18" s="3" t="n">
         <v>15.81</v>
       </c>
-      <c r="BZ18" s="3" t="n">
-        <v>15.81</v>
-      </c>
+      <c r="BZ18" s="3" t="n"/>
       <c r="CA18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB18" s="3" t="n"/>
+        <v>4.609</v>
+      </c>
+      <c r="CB18" s="3" t="n">
+        <v>4.639</v>
+      </c>
       <c r="CC18" s="3" t="n">
-        <v>4.609</v>
+        <v>4.607</v>
       </c>
       <c r="CD18" s="3" t="n">
-        <v>4.639</v>
-      </c>
-      <c r="CE18" s="3" t="n">
-        <v>4.607</v>
-      </c>
-      <c r="CF18" s="3" t="n">
         <v>4.617</v>
       </c>
-      <c r="CG18" s="3" t="n">
-        <v>4.617</v>
-      </c>
-      <c r="CH18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI18" s="3" t="n"/>
+      <c r="CE18" s="3" t="n"/>
+      <c r="CF18" s="4">
+        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG18" s="4">
+        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH18" s="4">
+        <f>IF(COUNT(BY18:BY23)=6,ROUND((BY18/BY23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI18" s="4">
+        <f>IF(COUNT(CG18:CG37)=20,IFERROR(ROUND(STDEV(CG18:CG37),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ18" s="4">
-        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK18" s="4">
-        <f>IF(COUNT(BY18:BY19)=2,ROUND((BY18/BY19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL18" s="4">
-        <f>IF(COUNT(BY18:BY23)=6,ROUND((BY18/BY23-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD18:CD19)=2,ROUND((CD18/CD19-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK18" s="5">
+        <f>IF(COUNT(CD18:CD19)=2,(CD18-CD19)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL18" s="3" t="n"/>
       <c r="CM18" s="4">
-        <f>IF(COUNT(CK18:CK37)=20,IFERROR(ROUND(STDEV(CK18:CK37),4),""),"")</f>
+        <f>IFERROR(X18-P18,"")</f>
         <v/>
       </c>
       <c r="CN18" s="4">
-        <f>IF(COUNT(CF18:CF19)=2,ROUND((CF18/CF19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO18" s="5">
-        <f>IF(COUNT(CF18:CF19)=2,(CF18-CF19)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP18" s="3" t="n"/>
+        <f>IFERROR(AF18-P18,"")</f>
+        <v/>
+      </c>
+      <c r="CO18" s="6">
+        <f>IF(COUNT(H18:H37)=20,IFERROR(CORREL(H18:H37,P18:P37),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP18" s="4">
+        <f>IFERROR(AN18-AV18,"")</f>
+        <v/>
+      </c>
       <c r="CQ18" s="4">
-        <f>IFERROR(X18-P18,"")</f>
-        <v/>
-      </c>
-      <c r="CR18" s="4">
-        <f>IFERROR(AF18-P18,"")</f>
-        <v/>
-      </c>
-      <c r="CS18" s="6">
-        <f>IF(COUNT(H18:H37)=20,IFERROR(CORREL(H18:H37,P18:P37),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT18" s="4">
-        <f>IFERROR(AN18-AV18,"")</f>
-        <v/>
-      </c>
-      <c r="CU18" s="4">
         <f>IFERROR(BD18-BL18,"")</f>
         <v/>
       </c>
-      <c r="CV18" s="6">
-        <f>BY18/CF18</f>
-        <v/>
-      </c>
-      <c r="CW18" s="4">
+      <c r="CR18" s="6">
+        <f>BY18/CD18</f>
+        <v/>
+      </c>
+      <c r="CS18" s="4">
         <f>IFERROR(P18-BT18,"")</f>
         <v/>
       </c>
@@ -2426,82 +2362,70 @@
       <c r="BY19" s="3" t="n">
         <v>16.5</v>
       </c>
-      <c r="BZ19" s="3" t="n">
-        <v>16.5</v>
-      </c>
+      <c r="BZ19" s="3" t="n"/>
       <c r="CA19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB19" s="3" t="n"/>
+        <v>4.665</v>
+      </c>
+      <c r="CB19" s="3" t="n">
+        <v>4.668</v>
+      </c>
       <c r="CC19" s="3" t="n">
-        <v>4.665</v>
+        <v>4.619</v>
       </c>
       <c r="CD19" s="3" t="n">
-        <v>4.668</v>
-      </c>
-      <c r="CE19" s="3" t="n">
-        <v>4.619</v>
-      </c>
-      <c r="CF19" s="3" t="n">
         <v>4.627</v>
       </c>
-      <c r="CG19" s="3" t="n">
-        <v>4.627</v>
-      </c>
-      <c r="CH19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI19" s="3" t="n"/>
+      <c r="CE19" s="3" t="n"/>
+      <c r="CF19" s="4">
+        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG19" s="4">
+        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH19" s="4">
+        <f>IF(COUNT(BY19:BY24)=6,ROUND((BY19/BY24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI19" s="4">
+        <f>IF(COUNT(CG19:CG38)=20,IFERROR(ROUND(STDEV(CG19:CG38),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ19" s="4">
-        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK19" s="4">
-        <f>IF(COUNT(BY19:BY20)=2,ROUND((BY19/BY20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL19" s="4">
-        <f>IF(COUNT(BY19:BY24)=6,ROUND((BY19/BY24-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD19:CD20)=2,ROUND((CD19/CD20-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK19" s="5">
+        <f>IF(COUNT(CD19:CD20)=2,(CD19-CD20)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL19" s="3" t="n"/>
       <c r="CM19" s="4">
-        <f>IF(COUNT(CK19:CK38)=20,IFERROR(ROUND(STDEV(CK19:CK38),4),""),"")</f>
+        <f>IFERROR(X19-P19,"")</f>
         <v/>
       </c>
       <c r="CN19" s="4">
-        <f>IF(COUNT(CF19:CF20)=2,ROUND((CF19/CF20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO19" s="5">
-        <f>IF(COUNT(CF19:CF20)=2,(CF19-CF20)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP19" s="3" t="n"/>
+        <f>IFERROR(AF19-P19,"")</f>
+        <v/>
+      </c>
+      <c r="CO19" s="6">
+        <f>IF(COUNT(H19:H38)=20,IFERROR(CORREL(H19:H38,P19:P38),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP19" s="4">
+        <f>IFERROR(AN19-AV19,"")</f>
+        <v/>
+      </c>
       <c r="CQ19" s="4">
-        <f>IFERROR(X19-P19,"")</f>
-        <v/>
-      </c>
-      <c r="CR19" s="4">
-        <f>IFERROR(AF19-P19,"")</f>
-        <v/>
-      </c>
-      <c r="CS19" s="6">
-        <f>IF(COUNT(H19:H38)=20,IFERROR(CORREL(H19:H38,P19:P38),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT19" s="4">
-        <f>IFERROR(AN19-AV19,"")</f>
-        <v/>
-      </c>
-      <c r="CU19" s="4">
         <f>IFERROR(BD19-BL19,"")</f>
         <v/>
       </c>
-      <c r="CV19" s="6">
-        <f>BY19/CF19</f>
-        <v/>
-      </c>
-      <c r="CW19" s="4">
+      <c r="CR19" s="6">
+        <f>BY19/CD19</f>
+        <v/>
+      </c>
+      <c r="CS19" s="4">
         <f>IFERROR(P19-BT19,"")</f>
         <v/>
       </c>
@@ -2731,82 +2655,70 @@
       <c r="BY20" s="3" t="n">
         <v>15.86</v>
       </c>
-      <c r="BZ20" s="3" t="n">
-        <v>15.86</v>
-      </c>
+      <c r="BZ20" s="3" t="n"/>
       <c r="CA20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB20" s="3" t="n"/>
+        <v>4.671</v>
+      </c>
+      <c r="CB20" s="3" t="n">
+        <v>4.702</v>
+      </c>
       <c r="CC20" s="3" t="n">
         <v>4.671</v>
       </c>
       <c r="CD20" s="3" t="n">
-        <v>4.702</v>
-      </c>
-      <c r="CE20" s="3" t="n">
-        <v>4.671</v>
-      </c>
-      <c r="CF20" s="3" t="n">
         <v>4.686</v>
       </c>
-      <c r="CG20" s="3" t="n">
-        <v>4.686</v>
-      </c>
-      <c r="CH20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI20" s="3" t="n"/>
+      <c r="CE20" s="3" t="n"/>
+      <c r="CF20" s="4">
+        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG20" s="4">
+        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH20" s="4">
+        <f>IF(COUNT(BY20:BY25)=6,ROUND((BY20/BY25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI20" s="4">
+        <f>IF(COUNT(CG20:CG39)=20,IFERROR(ROUND(STDEV(CG20:CG39),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ20" s="4">
-        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK20" s="4">
-        <f>IF(COUNT(BY20:BY21)=2,ROUND((BY20/BY21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL20" s="4">
-        <f>IF(COUNT(BY20:BY25)=6,ROUND((BY20/BY25-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD20:CD21)=2,ROUND((CD20/CD21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK20" s="5">
+        <f>IF(COUNT(CD20:CD21)=2,(CD20-CD21)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL20" s="3" t="n"/>
       <c r="CM20" s="4">
-        <f>IF(COUNT(CK20:CK39)=20,IFERROR(ROUND(STDEV(CK20:CK39),4),""),"")</f>
+        <f>IFERROR(X20-P20,"")</f>
         <v/>
       </c>
       <c r="CN20" s="4">
-        <f>IF(COUNT(CF20:CF21)=2,ROUND((CF20/CF21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO20" s="5">
-        <f>IF(COUNT(CF20:CF21)=2,(CF20-CF21)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP20" s="3" t="n"/>
+        <f>IFERROR(AF20-P20,"")</f>
+        <v/>
+      </c>
+      <c r="CO20" s="6">
+        <f>IF(COUNT(H20:H39)=20,IFERROR(CORREL(H20:H39,P20:P39),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP20" s="4">
+        <f>IFERROR(AN20-AV20,"")</f>
+        <v/>
+      </c>
       <c r="CQ20" s="4">
-        <f>IFERROR(X20-P20,"")</f>
-        <v/>
-      </c>
-      <c r="CR20" s="4">
-        <f>IFERROR(AF20-P20,"")</f>
-        <v/>
-      </c>
-      <c r="CS20" s="6">
-        <f>IF(COUNT(H20:H39)=20,IFERROR(CORREL(H20:H39,P20:P39),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT20" s="4">
-        <f>IFERROR(AN20-AV20,"")</f>
-        <v/>
-      </c>
-      <c r="CU20" s="4">
         <f>IFERROR(BD20-BL20,"")</f>
         <v/>
       </c>
-      <c r="CV20" s="6">
-        <f>BY20/CF20</f>
-        <v/>
-      </c>
-      <c r="CW20" s="4">
+      <c r="CR20" s="6">
+        <f>BY20/CD20</f>
+        <v/>
+      </c>
+      <c r="CS20" s="4">
         <f>IFERROR(P20-BT20,"")</f>
         <v/>
       </c>
@@ -3036,82 +2948,70 @@
       <c r="BY21" s="3" t="n">
         <v>15.99</v>
       </c>
-      <c r="BZ21" s="3" t="n">
-        <v>15.99</v>
-      </c>
+      <c r="BZ21" s="3" t="n"/>
       <c r="CA21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB21" s="3" t="n"/>
+        <v>4.684</v>
+      </c>
+      <c r="CB21" s="3" t="n">
+        <v>4.747</v>
+      </c>
       <c r="CC21" s="3" t="n">
-        <v>4.684</v>
+        <v>4.682</v>
       </c>
       <c r="CD21" s="3" t="n">
-        <v>4.747</v>
-      </c>
-      <c r="CE21" s="3" t="n">
-        <v>4.682</v>
-      </c>
-      <c r="CF21" s="3" t="n">
         <v>4.745</v>
       </c>
-      <c r="CG21" s="3" t="n">
-        <v>4.745</v>
-      </c>
-      <c r="CH21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI21" s="3" t="n"/>
+      <c r="CE21" s="3" t="n"/>
+      <c r="CF21" s="4">
+        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG21" s="4">
+        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH21" s="4">
+        <f>IF(COUNT(BY21:BY26)=6,ROUND((BY21/BY26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI21" s="4">
+        <f>IF(COUNT(CG21:CG40)=20,IFERROR(ROUND(STDEV(CG21:CG40),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ21" s="4">
-        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK21" s="4">
-        <f>IF(COUNT(BY21:BY22)=2,ROUND((BY21/BY22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL21" s="4">
-        <f>IF(COUNT(BY21:BY26)=6,ROUND((BY21/BY26-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD21:CD22)=2,ROUND((CD21/CD22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK21" s="5">
+        <f>IF(COUNT(CD21:CD22)=2,(CD21-CD22)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL21" s="3" t="n"/>
       <c r="CM21" s="4">
-        <f>IF(COUNT(CK21:CK40)=20,IFERROR(ROUND(STDEV(CK21:CK40),4),""),"")</f>
+        <f>IFERROR(X21-P21,"")</f>
         <v/>
       </c>
       <c r="CN21" s="4">
-        <f>IF(COUNT(CF21:CF22)=2,ROUND((CF21/CF22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO21" s="5">
-        <f>IF(COUNT(CF21:CF22)=2,(CF21-CF22)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP21" s="3" t="n"/>
+        <f>IFERROR(AF21-P21,"")</f>
+        <v/>
+      </c>
+      <c r="CO21" s="6">
+        <f>IF(COUNT(H21:H40)=20,IFERROR(CORREL(H21:H40,P21:P40),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP21" s="4">
+        <f>IFERROR(AN21-AV21,"")</f>
+        <v/>
+      </c>
       <c r="CQ21" s="4">
-        <f>IFERROR(X21-P21,"")</f>
-        <v/>
-      </c>
-      <c r="CR21" s="4">
-        <f>IFERROR(AF21-P21,"")</f>
-        <v/>
-      </c>
-      <c r="CS21" s="6">
-        <f>IF(COUNT(H21:H40)=20,IFERROR(CORREL(H21:H40,P21:P40),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT21" s="4">
-        <f>IFERROR(AN21-AV21,"")</f>
-        <v/>
-      </c>
-      <c r="CU21" s="4">
         <f>IFERROR(BD21-BL21,"")</f>
         <v/>
       </c>
-      <c r="CV21" s="6">
-        <f>BY21/CF21</f>
-        <v/>
-      </c>
-      <c r="CW21" s="4">
+      <c r="CR21" s="6">
+        <f>BY21/CD21</f>
+        <v/>
+      </c>
+      <c r="CS21" s="4">
         <f>IFERROR(P21-BT21,"")</f>
         <v/>
       </c>
@@ -3341,82 +3241,70 @@
       <c r="BY22" s="3" t="n">
         <v>17.09</v>
       </c>
-      <c r="BZ22" s="3" t="n">
-        <v>17.09</v>
-      </c>
+      <c r="BZ22" s="3" t="n"/>
       <c r="CA22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB22" s="3" t="n"/>
+        <v>4.669</v>
+      </c>
+      <c r="CB22" s="3" t="n">
+        <v>4.686</v>
+      </c>
       <c r="CC22" s="3" t="n">
-        <v>4.669</v>
+        <v>4.651</v>
       </c>
       <c r="CD22" s="3" t="n">
-        <v>4.686</v>
-      </c>
-      <c r="CE22" s="3" t="n">
-        <v>4.651</v>
-      </c>
-      <c r="CF22" s="3" t="n">
         <v>4.663</v>
       </c>
-      <c r="CG22" s="3" t="n">
-        <v>4.663</v>
-      </c>
-      <c r="CH22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI22" s="3" t="n"/>
+      <c r="CE22" s="3" t="n"/>
+      <c r="CF22" s="4">
+        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG22" s="4">
+        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH22" s="4">
+        <f>IF(COUNT(BY22:BY27)=6,ROUND((BY22/BY27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI22" s="4">
+        <f>IF(COUNT(CG22:CG41)=20,IFERROR(ROUND(STDEV(CG22:CG41),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ22" s="4">
-        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK22" s="4">
-        <f>IF(COUNT(BY22:BY23)=2,ROUND((BY22/BY23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL22" s="4">
-        <f>IF(COUNT(BY22:BY27)=6,ROUND((BY22/BY27-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD22:CD23)=2,ROUND((CD22/CD23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK22" s="5">
+        <f>IF(COUNT(CD22:CD23)=2,(CD22-CD23)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL22" s="3" t="n"/>
       <c r="CM22" s="4">
-        <f>IF(COUNT(CK22:CK41)=20,IFERROR(ROUND(STDEV(CK22:CK41),4),""),"")</f>
+        <f>IFERROR(X22-P22,"")</f>
         <v/>
       </c>
       <c r="CN22" s="4">
-        <f>IF(COUNT(CF22:CF23)=2,ROUND((CF22/CF23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO22" s="5">
-        <f>IF(COUNT(CF22:CF23)=2,(CF22-CF23)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP22" s="3" t="n"/>
+        <f>IFERROR(AF22-P22,"")</f>
+        <v/>
+      </c>
+      <c r="CO22" s="6">
+        <f>IF(COUNT(H22:H41)=20,IFERROR(CORREL(H22:H41,P22:P41),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP22" s="4">
+        <f>IFERROR(AN22-AV22,"")</f>
+        <v/>
+      </c>
       <c r="CQ22" s="4">
-        <f>IFERROR(X22-P22,"")</f>
-        <v/>
-      </c>
-      <c r="CR22" s="4">
-        <f>IFERROR(AF22-P22,"")</f>
-        <v/>
-      </c>
-      <c r="CS22" s="6">
-        <f>IF(COUNT(H22:H41)=20,IFERROR(CORREL(H22:H41,P22:P41),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT22" s="4">
-        <f>IFERROR(AN22-AV22,"")</f>
-        <v/>
-      </c>
-      <c r="CU22" s="4">
         <f>IFERROR(BD22-BL22,"")</f>
         <v/>
       </c>
-      <c r="CV22" s="6">
-        <f>BY22/CF22</f>
-        <v/>
-      </c>
-      <c r="CW22" s="4">
+      <c r="CR22" s="6">
+        <f>BY22/CD22</f>
+        <v/>
+      </c>
+      <c r="CS22" s="4">
         <f>IFERROR(P22-BT22,"")</f>
         <v/>
       </c>
@@ -3646,82 +3534,70 @@
       <c r="BY23" s="3" t="n">
         <v>20.66</v>
       </c>
-      <c r="BZ23" s="3" t="n">
-        <v>20.66</v>
-      </c>
+      <c r="BZ23" s="3" t="n"/>
       <c r="CA23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB23" s="3" t="n"/>
+        <v>4.637</v>
+      </c>
+      <c r="CB23" s="3" t="n">
+        <v>4.655</v>
+      </c>
       <c r="CC23" s="3" t="n">
-        <v>4.637</v>
+        <v>4.61</v>
       </c>
       <c r="CD23" s="3" t="n">
-        <v>4.655</v>
-      </c>
-      <c r="CE23" s="3" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="CF23" s="3" t="n">
         <v>4.622</v>
       </c>
-      <c r="CG23" s="3" t="n">
-        <v>4.622</v>
-      </c>
-      <c r="CH23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI23" s="3" t="n"/>
+      <c r="CE23" s="3" t="n"/>
+      <c r="CF23" s="4">
+        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG23" s="4">
+        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH23" s="4">
+        <f>IF(COUNT(BY23:BY28)=6,ROUND((BY23/BY28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI23" s="4">
+        <f>IF(COUNT(CG23:CG42)=20,IFERROR(ROUND(STDEV(CG23:CG42),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ23" s="4">
-        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK23" s="4">
-        <f>IF(COUNT(BY23:BY24)=2,ROUND((BY23/BY24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL23" s="4">
-        <f>IF(COUNT(BY23:BY28)=6,ROUND((BY23/BY28-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD23:CD24)=2,ROUND((CD23/CD24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK23" s="5">
+        <f>IF(COUNT(CD23:CD24)=2,(CD23-CD24)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL23" s="3" t="n"/>
       <c r="CM23" s="4">
-        <f>IF(COUNT(CK23:CK42)=20,IFERROR(ROUND(STDEV(CK23:CK42),4),""),"")</f>
+        <f>IFERROR(X23-P23,"")</f>
         <v/>
       </c>
       <c r="CN23" s="4">
-        <f>IF(COUNT(CF23:CF24)=2,ROUND((CF23/CF24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO23" s="5">
-        <f>IF(COUNT(CF23:CF24)=2,(CF23-CF24)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP23" s="3" t="n"/>
+        <f>IFERROR(AF23-P23,"")</f>
+        <v/>
+      </c>
+      <c r="CO23" s="6">
+        <f>IF(COUNT(H23:H42)=20,IFERROR(CORREL(H23:H42,P23:P42),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP23" s="4">
+        <f>IFERROR(AN23-AV23,"")</f>
+        <v/>
+      </c>
       <c r="CQ23" s="4">
-        <f>IFERROR(X23-P23,"")</f>
-        <v/>
-      </c>
-      <c r="CR23" s="4">
-        <f>IFERROR(AF23-P23,"")</f>
-        <v/>
-      </c>
-      <c r="CS23" s="6">
-        <f>IF(COUNT(H23:H42)=20,IFERROR(CORREL(H23:H42,P23:P42),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT23" s="4">
-        <f>IFERROR(AN23-AV23,"")</f>
-        <v/>
-      </c>
-      <c r="CU23" s="4">
         <f>IFERROR(BD23-BL23,"")</f>
         <v/>
       </c>
-      <c r="CV23" s="6">
-        <f>BY23/CF23</f>
-        <v/>
-      </c>
-      <c r="CW23" s="4">
+      <c r="CR23" s="6">
+        <f>BY23/CD23</f>
+        <v/>
+      </c>
+      <c r="CS23" s="4">
         <f>IFERROR(P23-BT23,"")</f>
         <v/>
       </c>
@@ -3951,82 +3827,70 @@
       <c r="BY24" s="3" t="n">
         <v>18.21</v>
       </c>
-      <c r="BZ24" s="3" t="n">
-        <v>18.21</v>
-      </c>
+      <c r="BZ24" s="3" t="n"/>
       <c r="CA24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB24" s="3" t="n"/>
+        <v>4.63</v>
+      </c>
+      <c r="CB24" s="3" t="n">
+        <v>4.635</v>
+      </c>
       <c r="CC24" s="3" t="n">
-        <v>4.63</v>
+        <v>4.588</v>
       </c>
       <c r="CD24" s="3" t="n">
-        <v>4.635</v>
-      </c>
-      <c r="CE24" s="3" t="n">
-        <v>4.588</v>
-      </c>
-      <c r="CF24" s="3" t="n">
         <v>4.604</v>
       </c>
-      <c r="CG24" s="3" t="n">
-        <v>4.604</v>
-      </c>
-      <c r="CH24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI24" s="3" t="n"/>
+      <c r="CE24" s="3" t="n"/>
+      <c r="CF24" s="4">
+        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG24" s="4">
+        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH24" s="4">
+        <f>IF(COUNT(BY24:BY29)=6,ROUND((BY24/BY29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI24" s="4">
+        <f>IF(COUNT(CG24:CG43)=20,IFERROR(ROUND(STDEV(CG24:CG43),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ24" s="4">
-        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK24" s="4">
-        <f>IF(COUNT(BY24:BY25)=2,ROUND((BY24/BY25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL24" s="4">
-        <f>IF(COUNT(BY24:BY29)=6,ROUND((BY24/BY29-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD24:CD25)=2,ROUND((CD24/CD25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK24" s="5">
+        <f>IF(COUNT(CD24:CD25)=2,(CD24-CD25)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL24" s="3" t="n"/>
       <c r="CM24" s="4">
-        <f>IF(COUNT(CK24:CK43)=20,IFERROR(ROUND(STDEV(CK24:CK43),4),""),"")</f>
+        <f>IFERROR(X24-P24,"")</f>
         <v/>
       </c>
       <c r="CN24" s="4">
-        <f>IF(COUNT(CF24:CF25)=2,ROUND((CF24/CF25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO24" s="5">
-        <f>IF(COUNT(CF24:CF25)=2,(CF24-CF25)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP24" s="3" t="n"/>
+        <f>IFERROR(AF24-P24,"")</f>
+        <v/>
+      </c>
+      <c r="CO24" s="6">
+        <f>IF(COUNT(H24:H43)=20,IFERROR(CORREL(H24:H43,P24:P43),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP24" s="4">
+        <f>IFERROR(AN24-AV24,"")</f>
+        <v/>
+      </c>
       <c r="CQ24" s="4">
-        <f>IFERROR(X24-P24,"")</f>
-        <v/>
-      </c>
-      <c r="CR24" s="4">
-        <f>IFERROR(AF24-P24,"")</f>
-        <v/>
-      </c>
-      <c r="CS24" s="6">
-        <f>IF(COUNT(H24:H43)=20,IFERROR(CORREL(H24:H43,P24:P43),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT24" s="4">
-        <f>IFERROR(AN24-AV24,"")</f>
-        <v/>
-      </c>
-      <c r="CU24" s="4">
         <f>IFERROR(BD24-BL24,"")</f>
         <v/>
       </c>
-      <c r="CV24" s="6">
-        <f>BY24/CF24</f>
-        <v/>
-      </c>
-      <c r="CW24" s="4">
+      <c r="CR24" s="6">
+        <f>BY24/CD24</f>
+        <v/>
+      </c>
+      <c r="CS24" s="4">
         <f>IFERROR(P24-BT24,"")</f>
         <v/>
       </c>
@@ -4256,82 +4120,70 @@
       <c r="BY25" s="3" t="n">
         <v>18.67</v>
       </c>
-      <c r="BZ25" s="3" t="n">
-        <v>18.67</v>
-      </c>
+      <c r="BZ25" s="3" t="n"/>
       <c r="CA25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB25" s="3" t="n"/>
+        <v>4.647</v>
+      </c>
+      <c r="CB25" s="3" t="n">
+        <v>4.665</v>
+      </c>
       <c r="CC25" s="3" t="n">
-        <v>4.647</v>
+        <v>4.63</v>
       </c>
       <c r="CD25" s="3" t="n">
-        <v>4.665</v>
-      </c>
-      <c r="CE25" s="3" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="CF25" s="3" t="n">
         <v>4.641</v>
       </c>
-      <c r="CG25" s="3" t="n">
-        <v>4.641</v>
-      </c>
-      <c r="CH25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI25" s="3" t="n"/>
+      <c r="CE25" s="3" t="n"/>
+      <c r="CF25" s="4">
+        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG25" s="4">
+        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH25" s="4">
+        <f>IF(COUNT(BY25:BY30)=6,ROUND((BY25/BY30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI25" s="4">
+        <f>IF(COUNT(CG25:CG44)=20,IFERROR(ROUND(STDEV(CG25:CG44),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ25" s="4">
-        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK25" s="4">
-        <f>IF(COUNT(BY25:BY26)=2,ROUND((BY25/BY26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL25" s="4">
-        <f>IF(COUNT(BY25:BY30)=6,ROUND((BY25/BY30-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD25:CD26)=2,ROUND((CD25/CD26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK25" s="5">
+        <f>IF(COUNT(CD25:CD26)=2,(CD25-CD26)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL25" s="3" t="n"/>
       <c r="CM25" s="4">
-        <f>IF(COUNT(CK25:CK44)=20,IFERROR(ROUND(STDEV(CK25:CK44),4),""),"")</f>
+        <f>IFERROR(X25-P25,"")</f>
         <v/>
       </c>
       <c r="CN25" s="4">
-        <f>IF(COUNT(CF25:CF26)=2,ROUND((CF25/CF26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO25" s="5">
-        <f>IF(COUNT(CF25:CF26)=2,(CF25-CF26)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP25" s="3" t="n"/>
+        <f>IFERROR(AF25-P25,"")</f>
+        <v/>
+      </c>
+      <c r="CO25" s="6">
+        <f>IF(COUNT(H25:H44)=20,IFERROR(CORREL(H25:H44,P25:P44),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP25" s="4">
+        <f>IFERROR(AN25-AV25,"")</f>
+        <v/>
+      </c>
       <c r="CQ25" s="4">
-        <f>IFERROR(X25-P25,"")</f>
-        <v/>
-      </c>
-      <c r="CR25" s="4">
-        <f>IFERROR(AF25-P25,"")</f>
-        <v/>
-      </c>
-      <c r="CS25" s="6">
-        <f>IF(COUNT(H25:H44)=20,IFERROR(CORREL(H25:H44,P25:P44),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT25" s="4">
-        <f>IFERROR(AN25-AV25,"")</f>
-        <v/>
-      </c>
-      <c r="CU25" s="4">
         <f>IFERROR(BD25-BL25,"")</f>
         <v/>
       </c>
-      <c r="CV25" s="6">
-        <f>BY25/CF25</f>
-        <v/>
-      </c>
-      <c r="CW25" s="4">
+      <c r="CR25" s="6">
+        <f>BY25/CD25</f>
+        <v/>
+      </c>
+      <c r="CS25" s="4">
         <f>IFERROR(P25-BT25,"")</f>
         <v/>
       </c>
@@ -4561,82 +4413,70 @@
       <c r="BY26" s="3" t="n">
         <v>18.58</v>
       </c>
-      <c r="BZ26" s="3" t="n">
-        <v>18.58</v>
-      </c>
+      <c r="BZ26" s="3" t="n"/>
       <c r="CA26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB26" s="3" t="n"/>
+        <v>4.683</v>
+      </c>
+      <c r="CB26" s="3" t="n">
+        <v>4.691</v>
+      </c>
       <c r="CC26" s="3" t="n">
-        <v>4.683</v>
+        <v>4.651</v>
       </c>
       <c r="CD26" s="3" t="n">
-        <v>4.691</v>
-      </c>
-      <c r="CE26" s="3" t="n">
-        <v>4.651</v>
-      </c>
-      <c r="CF26" s="3" t="n">
         <v>4.679</v>
       </c>
-      <c r="CG26" s="3" t="n">
-        <v>4.679</v>
-      </c>
-      <c r="CH26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI26" s="3" t="n"/>
+      <c r="CE26" s="3" t="n"/>
+      <c r="CF26" s="4">
+        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG26" s="4">
+        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH26" s="4">
+        <f>IF(COUNT(BY26:BY31)=6,ROUND((BY26/BY31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI26" s="4">
+        <f>IF(COUNT(CG26:CG45)=20,IFERROR(ROUND(STDEV(CG26:CG45),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ26" s="4">
-        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK26" s="4">
-        <f>IF(COUNT(BY26:BY27)=2,ROUND((BY26/BY27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL26" s="4">
-        <f>IF(COUNT(BY26:BY31)=6,ROUND((BY26/BY31-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD26:CD27)=2,ROUND((CD26/CD27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK26" s="5">
+        <f>IF(COUNT(CD26:CD27)=2,(CD26-CD27)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL26" s="3" t="n"/>
       <c r="CM26" s="4">
-        <f>IF(COUNT(CK26:CK45)=20,IFERROR(ROUND(STDEV(CK26:CK45),4),""),"")</f>
+        <f>IFERROR(X26-P26,"")</f>
         <v/>
       </c>
       <c r="CN26" s="4">
-        <f>IF(COUNT(CF26:CF27)=2,ROUND((CF26/CF27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO26" s="5">
-        <f>IF(COUNT(CF26:CF27)=2,(CF26-CF27)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP26" s="3" t="n"/>
+        <f>IFERROR(AF26-P26,"")</f>
+        <v/>
+      </c>
+      <c r="CO26" s="6">
+        <f>IF(COUNT(H26:H45)=20,IFERROR(CORREL(H26:H45,P26:P45),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP26" s="4">
+        <f>IFERROR(AN26-AV26,"")</f>
+        <v/>
+      </c>
       <c r="CQ26" s="4">
-        <f>IFERROR(X26-P26,"")</f>
-        <v/>
-      </c>
-      <c r="CR26" s="4">
-        <f>IFERROR(AF26-P26,"")</f>
-        <v/>
-      </c>
-      <c r="CS26" s="6">
-        <f>IF(COUNT(H26:H45)=20,IFERROR(CORREL(H26:H45,P26:P45),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT26" s="4">
-        <f>IFERROR(AN26-AV26,"")</f>
-        <v/>
-      </c>
-      <c r="CU26" s="4">
         <f>IFERROR(BD26-BL26,"")</f>
         <v/>
       </c>
-      <c r="CV26" s="6">
-        <f>BY26/CF26</f>
-        <v/>
-      </c>
-      <c r="CW26" s="4">
+      <c r="CR26" s="6">
+        <f>BY26/CD26</f>
+        <v/>
+      </c>
+      <c r="CS26" s="4">
         <f>IFERROR(P26-BT26,"")</f>
         <v/>
       </c>
@@ -4866,82 +4706,70 @@
       <c r="BY27" s="3" t="n">
         <v>18.7</v>
       </c>
-      <c r="BZ27" s="3" t="n">
-        <v>18.7</v>
-      </c>
+      <c r="BZ27" s="3" t="n"/>
       <c r="CA27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB27" s="3" t="n"/>
+        <v>4.699</v>
+      </c>
+      <c r="CB27" s="3" t="n">
+        <v>4.714</v>
+      </c>
       <c r="CC27" s="3" t="n">
-        <v>4.699</v>
+        <v>4.693</v>
       </c>
       <c r="CD27" s="3" t="n">
-        <v>4.714</v>
-      </c>
-      <c r="CE27" s="3" t="n">
-        <v>4.693</v>
-      </c>
-      <c r="CF27" s="3" t="n">
         <v>4.703</v>
       </c>
-      <c r="CG27" s="3" t="n">
-        <v>4.703</v>
-      </c>
-      <c r="CH27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI27" s="3" t="n"/>
+      <c r="CE27" s="3" t="n"/>
+      <c r="CF27" s="4">
+        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG27" s="4">
+        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH27" s="4">
+        <f>IF(COUNT(BY27:BY32)=6,ROUND((BY27/BY32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI27" s="4">
+        <f>IF(COUNT(CG27:CG46)=20,IFERROR(ROUND(STDEV(CG27:CG46),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ27" s="4">
-        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK27" s="4">
-        <f>IF(COUNT(BY27:BY28)=2,ROUND((BY27/BY28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL27" s="4">
-        <f>IF(COUNT(BY27:BY32)=6,ROUND((BY27/BY32-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD27:CD28)=2,ROUND((CD27/CD28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK27" s="5">
+        <f>IF(COUNT(CD27:CD28)=2,(CD27-CD28)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL27" s="3" t="n"/>
       <c r="CM27" s="4">
-        <f>IF(COUNT(CK27:CK46)=20,IFERROR(ROUND(STDEV(CK27:CK46),4),""),"")</f>
+        <f>IFERROR(X27-P27,"")</f>
         <v/>
       </c>
       <c r="CN27" s="4">
-        <f>IF(COUNT(CF27:CF28)=2,ROUND((CF27/CF28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO27" s="5">
-        <f>IF(COUNT(CF27:CF28)=2,(CF27-CF28)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP27" s="3" t="n"/>
+        <f>IFERROR(AF27-P27,"")</f>
+        <v/>
+      </c>
+      <c r="CO27" s="6">
+        <f>IF(COUNT(H27:H46)=20,IFERROR(CORREL(H27:H46,P27:P46),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP27" s="4">
+        <f>IFERROR(AN27-AV27,"")</f>
+        <v/>
+      </c>
       <c r="CQ27" s="4">
-        <f>IFERROR(X27-P27,"")</f>
-        <v/>
-      </c>
-      <c r="CR27" s="4">
-        <f>IFERROR(AF27-P27,"")</f>
-        <v/>
-      </c>
-      <c r="CS27" s="6">
-        <f>IF(COUNT(H27:H46)=20,IFERROR(CORREL(H27:H46,P27:P46),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT27" s="4">
-        <f>IFERROR(AN27-AV27,"")</f>
-        <v/>
-      </c>
-      <c r="CU27" s="4">
         <f>IFERROR(BD27-BL27,"")</f>
         <v/>
       </c>
-      <c r="CV27" s="6">
-        <f>BY27/CF27</f>
-        <v/>
-      </c>
-      <c r="CW27" s="4">
+      <c r="CR27" s="6">
+        <f>BY27/CD27</f>
+        <v/>
+      </c>
+      <c r="CS27" s="4">
         <f>IFERROR(P27-BT27,"")</f>
         <v/>
       </c>
@@ -5171,82 +4999,70 @@
       <c r="BY28" s="3" t="n">
         <v>16.64</v>
       </c>
-      <c r="BZ28" s="3" t="n">
-        <v>16.64</v>
-      </c>
+      <c r="BZ28" s="3" t="n"/>
       <c r="CA28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB28" s="3" t="n"/>
+        <v>4.64</v>
+      </c>
+      <c r="CB28" s="3" t="n">
+        <v>4.661</v>
+      </c>
       <c r="CC28" s="3" t="n">
-        <v>4.64</v>
+        <v>4.632</v>
       </c>
       <c r="CD28" s="3" t="n">
-        <v>4.661</v>
-      </c>
-      <c r="CE28" s="3" t="n">
-        <v>4.632</v>
-      </c>
-      <c r="CF28" s="3" t="n">
         <v>4.657</v>
       </c>
-      <c r="CG28" s="3" t="n">
-        <v>4.657</v>
-      </c>
-      <c r="CH28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI28" s="3" t="n"/>
+      <c r="CE28" s="3" t="n"/>
+      <c r="CF28" s="4">
+        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG28" s="4">
+        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH28" s="4">
+        <f>IF(COUNT(BY28:BY33)=6,ROUND((BY28/BY33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI28" s="4">
+        <f>IF(COUNT(CG28:CG47)=20,IFERROR(ROUND(STDEV(CG28:CG47),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ28" s="4">
-        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK28" s="4">
-        <f>IF(COUNT(BY28:BY29)=2,ROUND((BY28/BY29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL28" s="4">
-        <f>IF(COUNT(BY28:BY33)=6,ROUND((BY28/BY33-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD28:CD29)=2,ROUND((CD28/CD29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK28" s="5">
+        <f>IF(COUNT(CD28:CD29)=2,(CD28-CD29)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL28" s="3" t="n"/>
       <c r="CM28" s="4">
-        <f>IF(COUNT(CK28:CK47)=20,IFERROR(ROUND(STDEV(CK28:CK47),4),""),"")</f>
+        <f>IFERROR(X28-P28,"")</f>
         <v/>
       </c>
       <c r="CN28" s="4">
-        <f>IF(COUNT(CF28:CF29)=2,ROUND((CF28/CF29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO28" s="5">
-        <f>IF(COUNT(CF28:CF29)=2,(CF28-CF29)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP28" s="3" t="n"/>
+        <f>IFERROR(AF28-P28,"")</f>
+        <v/>
+      </c>
+      <c r="CO28" s="6">
+        <f>IF(COUNT(H28:H47)=20,IFERROR(CORREL(H28:H47,P28:P47),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP28" s="4">
+        <f>IFERROR(AN28-AV28,"")</f>
+        <v/>
+      </c>
       <c r="CQ28" s="4">
-        <f>IFERROR(X28-P28,"")</f>
-        <v/>
-      </c>
-      <c r="CR28" s="4">
-        <f>IFERROR(AF28-P28,"")</f>
-        <v/>
-      </c>
-      <c r="CS28" s="6">
-        <f>IF(COUNT(H28:H47)=20,IFERROR(CORREL(H28:H47,P28:P47),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT28" s="4">
-        <f>IFERROR(AN28-AV28,"")</f>
-        <v/>
-      </c>
-      <c r="CU28" s="4">
         <f>IFERROR(BD28-BL28,"")</f>
         <v/>
       </c>
-      <c r="CV28" s="6">
-        <f>BY28/CF28</f>
-        <v/>
-      </c>
-      <c r="CW28" s="4">
+      <c r="CR28" s="6">
+        <f>BY28/CD28</f>
+        <v/>
+      </c>
+      <c r="CS28" s="4">
         <f>IFERROR(P28-BT28,"")</f>
         <v/>
       </c>
@@ -5476,82 +5292,70 @@
       <c r="BY29" s="3" t="n">
         <v>17.05</v>
       </c>
-      <c r="BZ29" s="3" t="n">
-        <v>17.05</v>
-      </c>
+      <c r="BZ29" s="3" t="n"/>
       <c r="CA29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB29" s="3" t="n"/>
+        <v>4.6</v>
+      </c>
+      <c r="CB29" s="3" t="n">
+        <v>4.64</v>
+      </c>
       <c r="CC29" s="3" t="n">
-        <v>4.6</v>
+        <v>4.598</v>
       </c>
       <c r="CD29" s="3" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="CE29" s="3" t="n">
-        <v>4.598</v>
-      </c>
-      <c r="CF29" s="3" t="n">
         <v>4.628</v>
       </c>
-      <c r="CG29" s="3" t="n">
-        <v>4.628</v>
-      </c>
-      <c r="CH29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI29" s="3" t="n"/>
+      <c r="CE29" s="3" t="n"/>
+      <c r="CF29" s="4">
+        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG29" s="4">
+        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH29" s="4">
+        <f>IF(COUNT(BY29:BY34)=6,ROUND((BY29/BY34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI29" s="4">
+        <f>IF(COUNT(CG29:CG48)=20,IFERROR(ROUND(STDEV(CG29:CG48),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ29" s="4">
-        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK29" s="4">
-        <f>IF(COUNT(BY29:BY30)=2,ROUND((BY29/BY30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL29" s="4">
-        <f>IF(COUNT(BY29:BY34)=6,ROUND((BY29/BY34-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD29:CD30)=2,ROUND((CD29/CD30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK29" s="5">
+        <f>IF(COUNT(CD29:CD30)=2,(CD29-CD30)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL29" s="3" t="n"/>
       <c r="CM29" s="4">
-        <f>IF(COUNT(CK29:CK48)=20,IFERROR(ROUND(STDEV(CK29:CK48),4),""),"")</f>
+        <f>IFERROR(X29-P29,"")</f>
         <v/>
       </c>
       <c r="CN29" s="4">
-        <f>IF(COUNT(CF29:CF30)=2,ROUND((CF29/CF30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO29" s="5">
-        <f>IF(COUNT(CF29:CF30)=2,(CF29-CF30)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP29" s="3" t="n"/>
+        <f>IFERROR(AF29-P29,"")</f>
+        <v/>
+      </c>
+      <c r="CO29" s="6">
+        <f>IF(COUNT(H29:H48)=20,IFERROR(CORREL(H29:H48,P29:P48),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP29" s="4">
+        <f>IFERROR(AN29-AV29,"")</f>
+        <v/>
+      </c>
       <c r="CQ29" s="4">
-        <f>IFERROR(X29-P29,"")</f>
-        <v/>
-      </c>
-      <c r="CR29" s="4">
-        <f>IFERROR(AF29-P29,"")</f>
-        <v/>
-      </c>
-      <c r="CS29" s="6">
-        <f>IF(COUNT(H29:H48)=20,IFERROR(CORREL(H29:H48,P29:P48),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT29" s="4">
-        <f>IFERROR(AN29-AV29,"")</f>
-        <v/>
-      </c>
-      <c r="CU29" s="4">
         <f>IFERROR(BD29-BL29,"")</f>
         <v/>
       </c>
-      <c r="CV29" s="6">
-        <f>BY29/CF29</f>
-        <v/>
-      </c>
-      <c r="CW29" s="4">
+      <c r="CR29" s="6">
+        <f>BY29/CD29</f>
+        <v/>
+      </c>
+      <c r="CS29" s="4">
         <f>IFERROR(P29-BT29,"")</f>
         <v/>
       </c>
@@ -5781,82 +5585,70 @@
       <c r="BY30" s="3" t="n">
         <v>18.65</v>
       </c>
-      <c r="BZ30" s="3" t="n">
-        <v>18.65</v>
-      </c>
+      <c r="BZ30" s="3" t="n"/>
       <c r="CA30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB30" s="3" t="n"/>
+        <v>4.566</v>
+      </c>
+      <c r="CB30" s="3" t="n">
+        <v>4.608</v>
+      </c>
       <c r="CC30" s="3" t="n">
-        <v>4.566</v>
+        <v>4.56</v>
       </c>
       <c r="CD30" s="3" t="n">
-        <v>4.608</v>
-      </c>
-      <c r="CE30" s="3" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="CF30" s="3" t="n">
         <v>4.598</v>
       </c>
-      <c r="CG30" s="3" t="n">
-        <v>4.598</v>
-      </c>
-      <c r="CH30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI30" s="3" t="n"/>
+      <c r="CE30" s="3" t="n"/>
+      <c r="CF30" s="4">
+        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG30" s="4">
+        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH30" s="4">
+        <f>IF(COUNT(BY30:BY35)=6,ROUND((BY30/BY35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI30" s="4">
+        <f>IF(COUNT(CG30:CG49)=20,IFERROR(ROUND(STDEV(CG30:CG49),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ30" s="4">
-        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK30" s="4">
-        <f>IF(COUNT(BY30:BY31)=2,ROUND((BY30/BY31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL30" s="4">
-        <f>IF(COUNT(BY30:BY35)=6,ROUND((BY30/BY35-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD30:CD31)=2,ROUND((CD30/CD31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK30" s="5">
+        <f>IF(COUNT(CD30:CD31)=2,(CD30-CD31)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL30" s="3" t="n"/>
       <c r="CM30" s="4">
-        <f>IF(COUNT(CK30:CK49)=20,IFERROR(ROUND(STDEV(CK30:CK49),4),""),"")</f>
+        <f>IFERROR(X30-P30,"")</f>
         <v/>
       </c>
       <c r="CN30" s="4">
-        <f>IF(COUNT(CF30:CF31)=2,ROUND((CF30/CF31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO30" s="5">
-        <f>IF(COUNT(CF30:CF31)=2,(CF30-CF31)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP30" s="3" t="n"/>
+        <f>IFERROR(AF30-P30,"")</f>
+        <v/>
+      </c>
+      <c r="CO30" s="6">
+        <f>IF(COUNT(H30:H49)=20,IFERROR(CORREL(H30:H49,P30:P49),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP30" s="4">
+        <f>IFERROR(AN30-AV30,"")</f>
+        <v/>
+      </c>
       <c r="CQ30" s="4">
-        <f>IFERROR(X30-P30,"")</f>
-        <v/>
-      </c>
-      <c r="CR30" s="4">
-        <f>IFERROR(AF30-P30,"")</f>
-        <v/>
-      </c>
-      <c r="CS30" s="6">
-        <f>IF(COUNT(H30:H49)=20,IFERROR(CORREL(H30:H49,P30:P49),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT30" s="4">
-        <f>IFERROR(AN30-AV30,"")</f>
-        <v/>
-      </c>
-      <c r="CU30" s="4">
         <f>IFERROR(BD30-BL30,"")</f>
         <v/>
       </c>
-      <c r="CV30" s="6">
-        <f>BY30/CF30</f>
-        <v/>
-      </c>
-      <c r="CW30" s="4">
+      <c r="CR30" s="6">
+        <f>BY30/CD30</f>
+        <v/>
+      </c>
+      <c r="CS30" s="4">
         <f>IFERROR(P30-BT30,"")</f>
         <v/>
       </c>
@@ -6086,82 +5878,70 @@
       <c r="BY31" s="3" t="n">
         <v>18.77</v>
       </c>
-      <c r="BZ31" s="3" t="n">
-        <v>18.77</v>
-      </c>
+      <c r="BZ31" s="3" t="n"/>
       <c r="CA31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB31" s="3" t="n"/>
+        <v>4.521</v>
+      </c>
+      <c r="CB31" s="3" t="n">
+        <v>4.55</v>
+      </c>
       <c r="CC31" s="3" t="n">
-        <v>4.521</v>
+        <v>4.511</v>
       </c>
       <c r="CD31" s="3" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="CE31" s="3" t="n">
-        <v>4.511</v>
-      </c>
-      <c r="CF31" s="3" t="n">
         <v>4.541</v>
       </c>
-      <c r="CG31" s="3" t="n">
-        <v>4.541</v>
-      </c>
-      <c r="CH31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI31" s="3" t="n"/>
+      <c r="CE31" s="3" t="n"/>
+      <c r="CF31" s="4">
+        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG31" s="4">
+        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH31" s="4">
+        <f>IF(COUNT(BY31:BY36)=6,ROUND((BY31/BY36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI31" s="4">
+        <f>IF(COUNT(CG31:CG50)=20,IFERROR(ROUND(STDEV(CG31:CG50),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ31" s="4">
-        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK31" s="4">
-        <f>IF(COUNT(BY31:BY32)=2,ROUND((BY31/BY32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL31" s="4">
-        <f>IF(COUNT(BY31:BY36)=6,ROUND((BY31/BY36-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD31:CD32)=2,ROUND((CD31/CD32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK31" s="5">
+        <f>IF(COUNT(CD31:CD32)=2,(CD31-CD32)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL31" s="3" t="n"/>
       <c r="CM31" s="4">
-        <f>IF(COUNT(CK31:CK50)=20,IFERROR(ROUND(STDEV(CK31:CK50),4),""),"")</f>
+        <f>IFERROR(X31-P31,"")</f>
         <v/>
       </c>
       <c r="CN31" s="4">
-        <f>IF(COUNT(CF31:CF32)=2,ROUND((CF31/CF32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO31" s="5">
-        <f>IF(COUNT(CF31:CF32)=2,(CF31-CF32)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP31" s="3" t="n"/>
+        <f>IFERROR(AF31-P31,"")</f>
+        <v/>
+      </c>
+      <c r="CO31" s="6">
+        <f>IF(COUNT(H31:H50)=20,IFERROR(CORREL(H31:H50,P31:P50),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP31" s="4">
+        <f>IFERROR(AN31-AV31,"")</f>
+        <v/>
+      </c>
       <c r="CQ31" s="4">
-        <f>IFERROR(X31-P31,"")</f>
-        <v/>
-      </c>
-      <c r="CR31" s="4">
-        <f>IFERROR(AF31-P31,"")</f>
-        <v/>
-      </c>
-      <c r="CS31" s="6">
-        <f>IF(COUNT(H31:H50)=20,IFERROR(CORREL(H31:H50,P31:P50),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT31" s="4">
-        <f>IFERROR(AN31-AV31,"")</f>
-        <v/>
-      </c>
-      <c r="CU31" s="4">
         <f>IFERROR(BD31-BL31,"")</f>
         <v/>
       </c>
-      <c r="CV31" s="6">
-        <f>BY31/CF31</f>
-        <v/>
-      </c>
-      <c r="CW31" s="4">
+      <c r="CR31" s="6">
+        <f>BY31/CD31</f>
+        <v/>
+      </c>
+      <c r="CS31" s="4">
         <f>IFERROR(P31-BT31,"")</f>
         <v/>
       </c>
@@ -6391,82 +6171,70 @@
       <c r="BY32" s="3" t="n">
         <v>16.73</v>
       </c>
-      <c r="BZ32" s="3" t="n">
-        <v>16.73</v>
-      </c>
+      <c r="BZ32" s="3" t="n"/>
       <c r="CA32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB32" s="3" t="n"/>
+        <v>4.582</v>
+      </c>
+      <c r="CB32" s="3" t="n">
+        <v>4.596</v>
+      </c>
       <c r="CC32" s="3" t="n">
-        <v>4.582</v>
+        <v>4.561</v>
       </c>
       <c r="CD32" s="3" t="n">
-        <v>4.596</v>
-      </c>
-      <c r="CE32" s="3" t="n">
-        <v>4.561</v>
-      </c>
-      <c r="CF32" s="3" t="n">
         <v>4.569</v>
       </c>
-      <c r="CG32" s="3" t="n">
-        <v>4.569</v>
-      </c>
-      <c r="CH32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI32" s="3" t="n"/>
+      <c r="CE32" s="3" t="n"/>
+      <c r="CF32" s="4">
+        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG32" s="4">
+        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH32" s="4">
+        <f>IF(COUNT(BY32:BY37)=6,ROUND((BY32/BY37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI32" s="4">
+        <f>IF(COUNT(CG32:CG51)=20,IFERROR(ROUND(STDEV(CG32:CG51),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ32" s="4">
-        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK32" s="4">
-        <f>IF(COUNT(BY32:BY33)=2,ROUND((BY32/BY33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL32" s="4">
-        <f>IF(COUNT(BY32:BY37)=6,ROUND((BY32/BY37-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD32:CD33)=2,ROUND((CD32/CD33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK32" s="5">
+        <f>IF(COUNT(CD32:CD33)=2,(CD32-CD33)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL32" s="3" t="n"/>
       <c r="CM32" s="4">
-        <f>IF(COUNT(CK32:CK51)=20,IFERROR(ROUND(STDEV(CK32:CK51),4),""),"")</f>
+        <f>IFERROR(X32-P32,"")</f>
         <v/>
       </c>
       <c r="CN32" s="4">
-        <f>IF(COUNT(CF32:CF33)=2,ROUND((CF32/CF33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO32" s="5">
-        <f>IF(COUNT(CF32:CF33)=2,(CF32-CF33)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP32" s="3" t="n"/>
+        <f>IFERROR(AF32-P32,"")</f>
+        <v/>
+      </c>
+      <c r="CO32" s="6">
+        <f>IF(COUNT(H32:H51)=20,IFERROR(CORREL(H32:H51,P32:P51),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP32" s="4">
+        <f>IFERROR(AN32-AV32,"")</f>
+        <v/>
+      </c>
       <c r="CQ32" s="4">
-        <f>IFERROR(X32-P32,"")</f>
-        <v/>
-      </c>
-      <c r="CR32" s="4">
-        <f>IFERROR(AF32-P32,"")</f>
-        <v/>
-      </c>
-      <c r="CS32" s="6">
-        <f>IF(COUNT(H32:H51)=20,IFERROR(CORREL(H32:H51,P32:P51),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT32" s="4">
-        <f>IFERROR(AN32-AV32,"")</f>
-        <v/>
-      </c>
-      <c r="CU32" s="4">
         <f>IFERROR(BD32-BL32,"")</f>
         <v/>
       </c>
-      <c r="CV32" s="6">
-        <f>BY32/CF32</f>
-        <v/>
-      </c>
-      <c r="CW32" s="4">
+      <c r="CR32" s="6">
+        <f>BY32/CD32</f>
+        <v/>
+      </c>
+      <c r="CS32" s="4">
         <f>IFERROR(P32-BT32,"")</f>
         <v/>
       </c>
@@ -6696,82 +6464,70 @@
       <c r="BY33" s="3" t="n">
         <v>15.67</v>
       </c>
-      <c r="BZ33" s="3" t="n">
-        <v>15.67</v>
-      </c>
+      <c r="BZ33" s="3" t="n"/>
       <c r="CA33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB33" s="3" t="n"/>
+        <v>4.608</v>
+      </c>
+      <c r="CB33" s="3" t="n">
+        <v>4.61</v>
+      </c>
       <c r="CC33" s="3" t="n">
-        <v>4.608</v>
+        <v>4.539</v>
       </c>
       <c r="CD33" s="3" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="CE33" s="3" t="n">
-        <v>4.539</v>
-      </c>
-      <c r="CF33" s="3" t="n">
         <v>4.545</v>
       </c>
-      <c r="CG33" s="3" t="n">
-        <v>4.545</v>
-      </c>
-      <c r="CH33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI33" s="3" t="n"/>
+      <c r="CE33" s="3" t="n"/>
+      <c r="CF33" s="4">
+        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG33" s="4">
+        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH33" s="4">
+        <f>IF(COUNT(BY33:BY38)=6,ROUND((BY33/BY38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI33" s="4">
+        <f>IF(COUNT(CG33:CG52)=20,IFERROR(ROUND(STDEV(CG33:CG52),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ33" s="4">
-        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK33" s="4">
-        <f>IF(COUNT(BY33:BY34)=2,ROUND((BY33/BY34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL33" s="4">
-        <f>IF(COUNT(BY33:BY38)=6,ROUND((BY33/BY38-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD33:CD34)=2,ROUND((CD33/CD34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK33" s="5">
+        <f>IF(COUNT(CD33:CD34)=2,(CD33-CD34)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL33" s="3" t="n"/>
       <c r="CM33" s="4">
-        <f>IF(COUNT(CK33:CK52)=20,IFERROR(ROUND(STDEV(CK33:CK52),4),""),"")</f>
+        <f>IFERROR(X33-P33,"")</f>
         <v/>
       </c>
       <c r="CN33" s="4">
-        <f>IF(COUNT(CF33:CF34)=2,ROUND((CF33/CF34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO33" s="5">
-        <f>IF(COUNT(CF33:CF34)=2,(CF33-CF34)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP33" s="3" t="n"/>
+        <f>IFERROR(AF33-P33,"")</f>
+        <v/>
+      </c>
+      <c r="CO33" s="6">
+        <f>IF(COUNT(H33:H52)=20,IFERROR(CORREL(H33:H52,P33:P52),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP33" s="4">
+        <f>IFERROR(AN33-AV33,"")</f>
+        <v/>
+      </c>
       <c r="CQ33" s="4">
-        <f>IFERROR(X33-P33,"")</f>
-        <v/>
-      </c>
-      <c r="CR33" s="4">
-        <f>IFERROR(AF33-P33,"")</f>
-        <v/>
-      </c>
-      <c r="CS33" s="6">
-        <f>IF(COUNT(H33:H52)=20,IFERROR(CORREL(H33:H52,P33:P52),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT33" s="4">
-        <f>IFERROR(AN33-AV33,"")</f>
-        <v/>
-      </c>
-      <c r="CU33" s="4">
         <f>IFERROR(BD33-BL33,"")</f>
         <v/>
       </c>
-      <c r="CV33" s="6">
-        <f>BY33/CF33</f>
-        <v/>
-      </c>
-      <c r="CW33" s="4">
+      <c r="CR33" s="6">
+        <f>BY33/CD33</f>
+        <v/>
+      </c>
+      <c r="CS33" s="4">
         <f>IFERROR(P33-BT33,"")</f>
         <v/>
       </c>
@@ -7001,82 +6757,70 @@
       <c r="BY34" s="3" t="n">
         <v>16.5</v>
       </c>
-      <c r="BZ34" s="3" t="n">
-        <v>16.5</v>
-      </c>
+      <c r="BZ34" s="3" t="n"/>
       <c r="CA34" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB34" s="3" t="n"/>
+        <v>4.614</v>
+      </c>
+      <c r="CB34" s="3" t="n">
+        <v>4.614</v>
+      </c>
       <c r="CC34" s="3" t="n">
-        <v>4.614</v>
+        <v>4.525</v>
       </c>
       <c r="CD34" s="3" t="n">
-        <v>4.614</v>
-      </c>
-      <c r="CE34" s="3" t="n">
-        <v>4.525</v>
-      </c>
-      <c r="CF34" s="3" t="n">
         <v>4.585</v>
       </c>
-      <c r="CG34" s="3" t="n">
-        <v>4.585</v>
-      </c>
-      <c r="CH34" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI34" s="3" t="n"/>
+      <c r="CE34" s="3" t="n"/>
+      <c r="CF34" s="4">
+        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG34" s="4">
+        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH34" s="4">
+        <f>IF(COUNT(BY34:BY39)=6,ROUND((BY34/BY39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI34" s="4">
+        <f>IF(COUNT(CG34:CG53)=20,IFERROR(ROUND(STDEV(CG34:CG53),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ34" s="4">
-        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK34" s="4">
-        <f>IF(COUNT(BY34:BY35)=2,ROUND((BY34/BY35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL34" s="4">
-        <f>IF(COUNT(BY34:BY39)=6,ROUND((BY34/BY39-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD34:CD35)=2,ROUND((CD34/CD35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK34" s="5">
+        <f>IF(COUNT(CD34:CD35)=2,(CD34-CD35)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL34" s="3" t="n"/>
       <c r="CM34" s="4">
-        <f>IF(COUNT(CK34:CK53)=20,IFERROR(ROUND(STDEV(CK34:CK53),4),""),"")</f>
+        <f>IFERROR(X34-P34,"")</f>
         <v/>
       </c>
       <c r="CN34" s="4">
-        <f>IF(COUNT(CF34:CF35)=2,ROUND((CF34/CF35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO34" s="5">
-        <f>IF(COUNT(CF34:CF35)=2,(CF34-CF35)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP34" s="3" t="n"/>
+        <f>IFERROR(AF34-P34,"")</f>
+        <v/>
+      </c>
+      <c r="CO34" s="6">
+        <f>IF(COUNT(H34:H53)=20,IFERROR(CORREL(H34:H53,P34:P53),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP34" s="4">
+        <f>IFERROR(AN34-AV34,"")</f>
+        <v/>
+      </c>
       <c r="CQ34" s="4">
-        <f>IFERROR(X34-P34,"")</f>
-        <v/>
-      </c>
-      <c r="CR34" s="4">
-        <f>IFERROR(AF34-P34,"")</f>
-        <v/>
-      </c>
-      <c r="CS34" s="6">
-        <f>IF(COUNT(H34:H53)=20,IFERROR(CORREL(H34:H53,P34:P53),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT34" s="4">
-        <f>IFERROR(AN34-AV34,"")</f>
-        <v/>
-      </c>
-      <c r="CU34" s="4">
         <f>IFERROR(BD34-BL34,"")</f>
         <v/>
       </c>
-      <c r="CV34" s="6">
-        <f>BY34/CF34</f>
-        <v/>
-      </c>
-      <c r="CW34" s="4">
+      <c r="CR34" s="6">
+        <f>BY34/CD34</f>
+        <v/>
+      </c>
+      <c r="CS34" s="4">
         <f>IFERROR(P34-BT34,"")</f>
         <v/>
       </c>
@@ -7306,82 +7050,70 @@
       <c r="BY35" s="3" t="n">
         <v>17.16</v>
       </c>
-      <c r="BZ35" s="3" t="n">
-        <v>17.16</v>
-      </c>
+      <c r="BZ35" s="3" t="n"/>
       <c r="CA35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB35" s="3" t="n"/>
+        <v>4.585</v>
+      </c>
+      <c r="CB35" s="3" t="n">
+        <v>4.618</v>
+      </c>
       <c r="CC35" s="3" t="n">
-        <v>4.585</v>
+        <v>4.573</v>
       </c>
       <c r="CD35" s="3" t="n">
-        <v>4.618</v>
-      </c>
-      <c r="CE35" s="3" t="n">
-        <v>4.573</v>
-      </c>
-      <c r="CF35" s="3" t="n">
         <v>4.609</v>
       </c>
-      <c r="CG35" s="3" t="n">
-        <v>4.609</v>
-      </c>
-      <c r="CH35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI35" s="3" t="n"/>
+      <c r="CE35" s="3" t="n"/>
+      <c r="CF35" s="4">
+        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG35" s="4">
+        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH35" s="4">
+        <f>IF(COUNT(BY35:BY40)=6,ROUND((BY35/BY40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CI35" s="4">
+        <f>IF(COUNT(CG35:CG54)=20,IFERROR(ROUND(STDEV(CG35:CG54),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ35" s="4">
-        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK35" s="4">
-        <f>IF(COUNT(BY35:BY36)=2,ROUND((BY35/BY36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL35" s="4">
-        <f>IF(COUNT(BY35:BY40)=6,ROUND((BY35/BY40-1)*100,4),"")</f>
-        <v/>
-      </c>
+        <f>IF(COUNT(CD35:CD36)=2,ROUND((CD35/CD36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK35" s="5">
+        <f>IF(COUNT(CD35:CD36)=2,(CD35-CD36)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL35" s="3" t="n"/>
       <c r="CM35" s="4">
-        <f>IF(COUNT(CK35:CK54)=20,IFERROR(ROUND(STDEV(CK35:CK54),4),""),"")</f>
+        <f>IFERROR(X35-P35,"")</f>
         <v/>
       </c>
       <c r="CN35" s="4">
-        <f>IF(COUNT(CF35:CF36)=2,ROUND((CF35/CF36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO35" s="5">
-        <f>IF(COUNT(CF35:CF36)=2,(CF35-CF36)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP35" s="3" t="n"/>
+        <f>IFERROR(AF35-P35,"")</f>
+        <v/>
+      </c>
+      <c r="CO35" s="6">
+        <f>IF(COUNT(H35:H54)=20,IFERROR(CORREL(H35:H54,P35:P54),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP35" s="4">
+        <f>IFERROR(AN35-AV35,"")</f>
+        <v/>
+      </c>
       <c r="CQ35" s="4">
-        <f>IFERROR(X35-P35,"")</f>
-        <v/>
-      </c>
-      <c r="CR35" s="4">
-        <f>IFERROR(AF35-P35,"")</f>
-        <v/>
-      </c>
-      <c r="CS35" s="6">
-        <f>IF(COUNT(H35:H54)=20,IFERROR(CORREL(H35:H54,P35:P54),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT35" s="4">
-        <f>IFERROR(AN35-AV35,"")</f>
-        <v/>
-      </c>
-      <c r="CU35" s="4">
         <f>IFERROR(BD35-BL35,"")</f>
         <v/>
       </c>
-      <c r="CV35" s="6">
-        <f>BY35/CF35</f>
-        <v/>
-      </c>
-      <c r="CW35" s="4">
+      <c r="CR35" s="6">
+        <f>BY35/CD35</f>
+        <v/>
+      </c>
+      <c r="CS35" s="4">
         <f>IFERROR(P35-BT35,"")</f>
         <v/>
       </c>
@@ -7611,79 +7343,67 @@
       <c r="BY36" s="3" t="n">
         <v>15.03</v>
       </c>
-      <c r="BZ36" s="3" t="n">
-        <v>15.03</v>
-      </c>
+      <c r="BZ36" s="3" t="n"/>
       <c r="CA36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB36" s="3" t="n"/>
+        <v>4.541</v>
+      </c>
+      <c r="CB36" s="3" t="n">
+        <v>4.571</v>
+      </c>
       <c r="CC36" s="3" t="n">
-        <v>4.541</v>
+        <v>4.539</v>
       </c>
       <c r="CD36" s="3" t="n">
-        <v>4.571</v>
-      </c>
-      <c r="CE36" s="3" t="n">
-        <v>4.539</v>
-      </c>
-      <c r="CF36" s="3" t="n">
         <v>4.569</v>
       </c>
-      <c r="CG36" s="3" t="n">
-        <v>4.569</v>
-      </c>
-      <c r="CH36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI36" s="3" t="n"/>
+      <c r="CE36" s="3" t="n"/>
+      <c r="CF36" s="4">
+        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG36" s="4">
+        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH36" s="4" t="n"/>
+      <c r="CI36" s="4">
+        <f>IF(COUNT(CG36:CG55)=20,IFERROR(ROUND(STDEV(CG36:CG55),4),""),"")</f>
+        <v/>
+      </c>
       <c r="CJ36" s="4">
-        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK36" s="4">
-        <f>IF(COUNT(BY36:BY37)=2,ROUND((BY36/BY37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL36" s="4" t="n"/>
+        <f>IF(COUNT(CD36:CD37)=2,ROUND((CD36/CD37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK36" s="5">
+        <f>IF(COUNT(CD36:CD37)=2,(CD36-CD37)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL36" s="3" t="n"/>
       <c r="CM36" s="4">
-        <f>IF(COUNT(CK36:CK55)=20,IFERROR(ROUND(STDEV(CK36:CK55),4),""),"")</f>
+        <f>IFERROR(X36-P36,"")</f>
         <v/>
       </c>
       <c r="CN36" s="4">
-        <f>IF(COUNT(CF36:CF37)=2,ROUND((CF36/CF37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO36" s="5">
-        <f>IF(COUNT(CF36:CF37)=2,(CF36-CF37)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP36" s="3" t="n"/>
+        <f>IFERROR(AF36-P36,"")</f>
+        <v/>
+      </c>
+      <c r="CO36" s="6">
+        <f>IF(COUNT(H36:H55)=20,IFERROR(CORREL(H36:H55,P36:P55),""),"")</f>
+        <v/>
+      </c>
+      <c r="CP36" s="4">
+        <f>IFERROR(AN36-AV36,"")</f>
+        <v/>
+      </c>
       <c r="CQ36" s="4">
-        <f>IFERROR(X36-P36,"")</f>
-        <v/>
-      </c>
-      <c r="CR36" s="4">
-        <f>IFERROR(AF36-P36,"")</f>
-        <v/>
-      </c>
-      <c r="CS36" s="6">
-        <f>IF(COUNT(H36:H55)=20,IFERROR(CORREL(H36:H55,P36:P55),""),"")</f>
-        <v/>
-      </c>
-      <c r="CT36" s="4">
-        <f>IFERROR(AN36-AV36,"")</f>
-        <v/>
-      </c>
-      <c r="CU36" s="4">
         <f>IFERROR(BD36-BL36,"")</f>
         <v/>
       </c>
-      <c r="CV36" s="6">
-        <f>BY36/CF36</f>
-        <v/>
-      </c>
-      <c r="CW36" s="4">
+      <c r="CR36" s="6">
+        <f>BY36/CD36</f>
+        <v/>
+      </c>
+      <c r="CS36" s="4">
         <f>IFERROR(P36-BT36,"")</f>
         <v/>
       </c>
@@ -7913,73 +7633,61 @@
       <c r="BY37" s="3" t="n">
         <v>15.84</v>
       </c>
-      <c r="BZ37" s="3" t="n">
-        <v>15.84</v>
-      </c>
+      <c r="BZ37" s="3" t="n"/>
       <c r="CA37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB37" s="3" t="n"/>
+        <v>4.577</v>
+      </c>
+      <c r="CB37" s="3" t="n">
+        <v>4.581</v>
+      </c>
       <c r="CC37" s="3" t="n">
-        <v>4.577</v>
+        <v>4.529</v>
       </c>
       <c r="CD37" s="3" t="n">
-        <v>4.581</v>
-      </c>
-      <c r="CE37" s="3" t="n">
-        <v>4.529</v>
-      </c>
-      <c r="CF37" s="3" t="n">
         <v>4.539</v>
       </c>
-      <c r="CG37" s="3" t="n">
-        <v>4.539</v>
-      </c>
-      <c r="CH37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI37" s="3" t="n"/>
+      <c r="CE37" s="3" t="n"/>
+      <c r="CF37" s="4">
+        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG37" s="4">
+        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH37" s="4" t="n"/>
+      <c r="CI37" s="4" t="n"/>
       <c r="CJ37" s="4">
-        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK37" s="4">
-        <f>IF(COUNT(BY37:BY38)=2,ROUND((BY37/BY38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL37" s="4" t="n"/>
-      <c r="CM37" s="4" t="n"/>
+        <f>IF(COUNT(CD37:CD38)=2,ROUND((CD37/CD38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK37" s="5">
+        <f>IF(COUNT(CD37:CD38)=2,(CD37-CD38)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL37" s="3" t="n"/>
+      <c r="CM37" s="4">
+        <f>IFERROR(X37-P37,"")</f>
+        <v/>
+      </c>
       <c r="CN37" s="4">
-        <f>IF(COUNT(CF37:CF38)=2,ROUND((CF37/CF38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO37" s="5">
-        <f>IF(COUNT(CF37:CF38)=2,(CF37-CF38)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP37" s="3" t="n"/>
+        <f>IFERROR(AF37-P37,"")</f>
+        <v/>
+      </c>
+      <c r="CO37" s="6" t="n"/>
+      <c r="CP37" s="4">
+        <f>IFERROR(AN37-AV37,"")</f>
+        <v/>
+      </c>
       <c r="CQ37" s="4">
-        <f>IFERROR(X37-P37,"")</f>
-        <v/>
-      </c>
-      <c r="CR37" s="4">
-        <f>IFERROR(AF37-P37,"")</f>
-        <v/>
-      </c>
-      <c r="CS37" s="6" t="n"/>
-      <c r="CT37" s="4">
-        <f>IFERROR(AN37-AV37,"")</f>
-        <v/>
-      </c>
-      <c r="CU37" s="4">
         <f>IFERROR(BD37-BL37,"")</f>
         <v/>
       </c>
-      <c r="CV37" s="6">
-        <f>BY37/CF37</f>
-        <v/>
-      </c>
-      <c r="CW37" s="4">
+      <c r="CR37" s="6">
+        <f>BY37/CD37</f>
+        <v/>
+      </c>
+      <c r="CS37" s="4">
         <f>IFERROR(P37-BT37,"")</f>
         <v/>
       </c>
@@ -8209,73 +7917,61 @@
       <c r="BY38" s="3" t="n">
         <v>16.9</v>
       </c>
-      <c r="BZ38" s="3" t="n">
-        <v>16.9</v>
-      </c>
+      <c r="BZ38" s="3" t="n"/>
       <c r="CA38" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB38" s="3" t="n"/>
+        <v>4.561</v>
+      </c>
+      <c r="CB38" s="3" t="n">
+        <v>4.597</v>
+      </c>
       <c r="CC38" s="3" t="n">
-        <v>4.561</v>
+        <v>4.557</v>
       </c>
       <c r="CD38" s="3" t="n">
-        <v>4.597</v>
-      </c>
-      <c r="CE38" s="3" t="n">
-        <v>4.557</v>
-      </c>
-      <c r="CF38" s="3" t="n">
         <v>4.569</v>
       </c>
-      <c r="CG38" s="3" t="n">
-        <v>4.569</v>
-      </c>
-      <c r="CH38" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI38" s="3" t="n"/>
+      <c r="CE38" s="3" t="n"/>
+      <c r="CF38" s="4">
+        <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG38" s="4">
+        <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH38" s="4" t="n"/>
+      <c r="CI38" s="4" t="n"/>
       <c r="CJ38" s="4">
-        <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK38" s="4">
-        <f>IF(COUNT(BY38:BY39)=2,ROUND((BY38/BY39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL38" s="4" t="n"/>
-      <c r="CM38" s="4" t="n"/>
+        <f>IF(COUNT(CD38:CD39)=2,ROUND((CD38/CD39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK38" s="5">
+        <f>IF(COUNT(CD38:CD39)=2,(CD38-CD39)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL38" s="3" t="n"/>
+      <c r="CM38" s="4">
+        <f>IFERROR(X38-P38,"")</f>
+        <v/>
+      </c>
       <c r="CN38" s="4">
-        <f>IF(COUNT(CF38:CF39)=2,ROUND((CF38/CF39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO38" s="5">
-        <f>IF(COUNT(CF38:CF39)=2,(CF38-CF39)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP38" s="3" t="n"/>
+        <f>IFERROR(AF38-P38,"")</f>
+        <v/>
+      </c>
+      <c r="CO38" s="6" t="n"/>
+      <c r="CP38" s="4">
+        <f>IFERROR(AN38-AV38,"")</f>
+        <v/>
+      </c>
       <c r="CQ38" s="4">
-        <f>IFERROR(X38-P38,"")</f>
-        <v/>
-      </c>
-      <c r="CR38" s="4">
-        <f>IFERROR(AF38-P38,"")</f>
-        <v/>
-      </c>
-      <c r="CS38" s="6" t="n"/>
-      <c r="CT38" s="4">
-        <f>IFERROR(AN38-AV38,"")</f>
-        <v/>
-      </c>
-      <c r="CU38" s="4">
         <f>IFERROR(BD38-BL38,"")</f>
         <v/>
       </c>
-      <c r="CV38" s="6">
-        <f>BY38/CF38</f>
-        <v/>
-      </c>
-      <c r="CW38" s="4">
+      <c r="CR38" s="6">
+        <f>BY38/CD38</f>
+        <v/>
+      </c>
+      <c r="CS38" s="4">
         <f>IFERROR(P38-BT38,"")</f>
         <v/>
       </c>
@@ -8505,73 +8201,61 @@
       <c r="BY39" s="3" t="n">
         <v>16.13</v>
       </c>
-      <c r="BZ39" s="3" t="n">
-        <v>16.13</v>
-      </c>
+      <c r="BZ39" s="3" t="n"/>
       <c r="CA39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB39" s="3" t="n"/>
+        <v>4.497</v>
+      </c>
+      <c r="CB39" s="3" t="n">
+        <v>4.533</v>
+      </c>
       <c r="CC39" s="3" t="n">
-        <v>4.497</v>
+        <v>4.485</v>
       </c>
       <c r="CD39" s="3" t="n">
-        <v>4.533</v>
-      </c>
-      <c r="CE39" s="3" t="n">
-        <v>4.485</v>
-      </c>
-      <c r="CF39" s="3" t="n">
         <v>4.529</v>
       </c>
-      <c r="CG39" s="3" t="n">
-        <v>4.529</v>
-      </c>
-      <c r="CH39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI39" s="3" t="n"/>
+      <c r="CE39" s="3" t="n"/>
+      <c r="CF39" s="4">
+        <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG39" s="4">
+        <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH39" s="4" t="n"/>
+      <c r="CI39" s="4" t="n"/>
       <c r="CJ39" s="4">
-        <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK39" s="4">
-        <f>IF(COUNT(BY39:BY40)=2,ROUND((BY39/BY40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL39" s="4" t="n"/>
-      <c r="CM39" s="4" t="n"/>
+        <f>IF(COUNT(CD39:CD40)=2,ROUND((CD39/CD40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK39" s="5">
+        <f>IF(COUNT(CD39:CD40)=2,(CD39-CD40)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL39" s="3" t="n"/>
+      <c r="CM39" s="4">
+        <f>IFERROR(X39-P39,"")</f>
+        <v/>
+      </c>
       <c r="CN39" s="4">
-        <f>IF(COUNT(CF39:CF40)=2,ROUND((CF39/CF40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO39" s="5">
-        <f>IF(COUNT(CF39:CF40)=2,(CF39-CF40)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP39" s="3" t="n"/>
+        <f>IFERROR(AF39-P39,"")</f>
+        <v/>
+      </c>
+      <c r="CO39" s="6" t="n"/>
+      <c r="CP39" s="4">
+        <f>IFERROR(AN39-AV39,"")</f>
+        <v/>
+      </c>
       <c r="CQ39" s="4">
-        <f>IFERROR(X39-P39,"")</f>
-        <v/>
-      </c>
-      <c r="CR39" s="4">
-        <f>IFERROR(AF39-P39,"")</f>
-        <v/>
-      </c>
-      <c r="CS39" s="6" t="n"/>
-      <c r="CT39" s="4">
-        <f>IFERROR(AN39-AV39,"")</f>
-        <v/>
-      </c>
-      <c r="CU39" s="4">
         <f>IFERROR(BD39-BL39,"")</f>
         <v/>
       </c>
-      <c r="CV39" s="6">
-        <f>BY39/CF39</f>
-        <v/>
-      </c>
-      <c r="CW39" s="4">
+      <c r="CR39" s="6">
+        <f>BY39/CD39</f>
+        <v/>
+      </c>
+      <c r="CS39" s="4">
         <f>IFERROR(P39-BT39,"")</f>
         <v/>
       </c>
@@ -8774,73 +8458,61 @@
       <c r="BY40" s="3" t="n">
         <v>15.57</v>
       </c>
-      <c r="BZ40" s="3" t="n">
-        <v>15.57</v>
-      </c>
+      <c r="BZ40" s="3" t="n"/>
       <c r="CA40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB40" s="3" t="n"/>
+        <v>4.457</v>
+      </c>
+      <c r="CB40" s="3" t="n">
+        <v>4.491</v>
+      </c>
       <c r="CC40" s="3" t="n">
         <v>4.457</v>
       </c>
       <c r="CD40" s="3" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="CE40" s="3" t="n">
-        <v>4.457</v>
-      </c>
-      <c r="CF40" s="3" t="n">
         <v>4.479</v>
       </c>
-      <c r="CG40" s="3" t="n">
-        <v>4.479</v>
-      </c>
-      <c r="CH40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI40" s="3" t="n"/>
+      <c r="CE40" s="3" t="n"/>
+      <c r="CF40" s="4">
+        <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CG40" s="4">
+        <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CH40" s="4" t="n"/>
+      <c r="CI40" s="4" t="n"/>
       <c r="CJ40" s="4">
-        <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CK40" s="4">
-        <f>IF(COUNT(BY40:BY41)=2,ROUND((BY40/BY41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CL40" s="4" t="n"/>
-      <c r="CM40" s="4" t="n"/>
+        <f>IF(COUNT(CD40:CD41)=2,ROUND((CD40/CD41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="CK40" s="5">
+        <f>IF(COUNT(CD40:CD41)=2,(CD40-CD41)*100,"")</f>
+        <v/>
+      </c>
+      <c r="CL40" s="3" t="n"/>
+      <c r="CM40" s="4">
+        <f>IFERROR(X40-P40,"")</f>
+        <v/>
+      </c>
       <c r="CN40" s="4">
-        <f>IF(COUNT(CF40:CF41)=2,ROUND((CF40/CF41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="CO40" s="5">
-        <f>IF(COUNT(CF40:CF41)=2,(CF40-CF41)*100,"")</f>
-        <v/>
-      </c>
-      <c r="CP40" s="3" t="n"/>
+        <f>IFERROR(AF40-P40,"")</f>
+        <v/>
+      </c>
+      <c r="CO40" s="6" t="n"/>
+      <c r="CP40" s="4">
+        <f>IFERROR(AN40-AV40,"")</f>
+        <v/>
+      </c>
       <c r="CQ40" s="4">
-        <f>IFERROR(X40-P40,"")</f>
-        <v/>
-      </c>
-      <c r="CR40" s="4">
-        <f>IFERROR(AF40-P40,"")</f>
-        <v/>
-      </c>
-      <c r="CS40" s="6" t="n"/>
-      <c r="CT40" s="4">
-        <f>IFERROR(AN40-AV40,"")</f>
-        <v/>
-      </c>
-      <c r="CU40" s="4">
         <f>IFERROR(BD40-BL40,"")</f>
         <v/>
       </c>
-      <c r="CV40" s="6">
-        <f>BY40/CF40</f>
-        <v/>
-      </c>
-      <c r="CW40" s="4">
+      <c r="CR40" s="6">
+        <f>BY40/CD40</f>
+        <v/>
+      </c>
+      <c r="CS40" s="4">
         <f>IFERROR(P40-BT40,"")</f>
         <v/>
       </c>

</xml_diff>